<commit_message>
Refactor NutrimentalExporter: Update image handling for seals, improve centering logic, and adjust sizes for better layout in Excel output
</commit_message>
<xml_diff>
--- a/templates/formato.xlsx
+++ b/templates/formato.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29029"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29127"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/e039d0c270e9facf/Desktop/Developer/UANL---LABORATORIO-DE-ALIMENTOS-MEDICAMENTOS-Y-TOXICOLOGIA/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/e039d0c270e9facf/Desktop/Developer/UANL---LABORATORIO-DE-ALIMENTOS-MEDICAMENTOS-Y-TOXICOLOGIA/templates/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="101" documentId="8_{47FAC42F-AC07-43D6-8172-01CEADEBF0F6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{916F2CCF-DC7F-4EEF-8AE2-D0D5A0F8E5EE}"/>
+  <xr:revisionPtr revIDLastSave="103" documentId="8_{47FAC42F-AC07-43D6-8172-01CEADEBF0F6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{2716931A-8BFA-4F91-B0C5-888B0B410AC4}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{1CB8A4CE-E91B-448F-9BE6-E546BA7C8907}"/>
   </bookViews>
@@ -386,6 +386,27 @@
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
@@ -416,29 +437,8 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -582,10 +582,6 @@
     <xdr:clientData/>
   </xdr:twoCellAnchor>
 </xdr:wsDr>
-</file>
-
-<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
-<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -921,28 +917,28 @@
   </cols>
   <sheetData>
     <row r="4" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A4" s="28"/>
-      <c r="B4" s="28"/>
-      <c r="C4" s="28"/>
-      <c r="D4" s="28"/>
-      <c r="E4" s="28"/>
-      <c r="F4" s="28"/>
-      <c r="G4" s="28"/>
-      <c r="H4" s="28"/>
-      <c r="I4" s="28"/>
-      <c r="J4" s="28"/>
+      <c r="A4" s="35"/>
+      <c r="B4" s="35"/>
+      <c r="C4" s="35"/>
+      <c r="D4" s="35"/>
+      <c r="E4" s="35"/>
+      <c r="F4" s="35"/>
+      <c r="G4" s="35"/>
+      <c r="H4" s="35"/>
+      <c r="I4" s="35"/>
+      <c r="J4" s="35"/>
     </row>
     <row r="5" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A5" s="28"/>
-      <c r="B5" s="28"/>
-      <c r="C5" s="28"/>
-      <c r="D5" s="28"/>
-      <c r="E5" s="28"/>
-      <c r="F5" s="28"/>
-      <c r="G5" s="28"/>
-      <c r="H5" s="28"/>
-      <c r="I5" s="28"/>
-      <c r="J5" s="28"/>
+      <c r="A5" s="35"/>
+      <c r="B5" s="35"/>
+      <c r="C5" s="35"/>
+      <c r="D5" s="35"/>
+      <c r="E5" s="35"/>
+      <c r="F5" s="35"/>
+      <c r="G5" s="35"/>
+      <c r="H5" s="35"/>
+      <c r="I5" s="35"/>
+      <c r="J5" s="35"/>
     </row>
     <row r="6" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A6" s="1"/>
@@ -982,25 +978,25 @@
       <c r="J8" s="2"/>
     </row>
     <row r="10" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="B10" s="29" t="s">
+      <c r="B10" s="36" t="s">
         <v>0</v>
       </c>
-      <c r="C10" s="29"/>
-      <c r="D10" s="29"/>
-      <c r="E10" s="29"/>
-      <c r="F10" s="29"/>
-      <c r="G10" s="29"/>
-      <c r="H10" s="29"/>
-      <c r="I10" s="29"/>
-      <c r="J10" s="29"/>
+      <c r="C10" s="36"/>
+      <c r="D10" s="36"/>
+      <c r="E10" s="36"/>
+      <c r="F10" s="36"/>
+      <c r="G10" s="36"/>
+      <c r="H10" s="36"/>
+      <c r="I10" s="36"/>
+      <c r="J10" s="36"/>
     </row>
     <row r="12" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="B12" s="25" t="s">
+      <c r="B12" s="32" t="s">
         <v>18</v>
       </c>
-      <c r="C12" s="25"/>
-      <c r="D12" s="25"/>
-      <c r="E12" s="25"/>
+      <c r="C12" s="32"/>
+      <c r="D12" s="32"/>
+      <c r="E12" s="32"/>
     </row>
     <row r="13" spans="1:10" ht="15" thickBot="1" x14ac:dyDescent="0.35"/>
     <row r="14" spans="1:10" x14ac:dyDescent="0.3">
@@ -1015,17 +1011,17 @@
       <c r="J14" s="7"/>
     </row>
     <row r="15" spans="1:10" ht="21" x14ac:dyDescent="0.4">
-      <c r="B15" s="40" t="s">
+      <c r="B15" s="29" t="s">
         <v>10</v>
       </c>
-      <c r="C15" s="41"/>
-      <c r="D15" s="41"/>
-      <c r="E15" s="41"/>
-      <c r="F15" s="41"/>
-      <c r="G15" s="41"/>
-      <c r="H15" s="41"/>
-      <c r="I15" s="41"/>
-      <c r="J15" s="42"/>
+      <c r="C15" s="30"/>
+      <c r="D15" s="30"/>
+      <c r="E15" s="30"/>
+      <c r="F15" s="30"/>
+      <c r="G15" s="30"/>
+      <c r="H15" s="30"/>
+      <c r="I15" s="30"/>
+      <c r="J15" s="31"/>
     </row>
     <row r="16" spans="1:10" x14ac:dyDescent="0.3">
       <c r="B16" s="3"/>
@@ -1074,23 +1070,23 @@
       <c r="C20" s="10"/>
       <c r="D20" s="10"/>
       <c r="E20" s="10"/>
-      <c r="F20" s="38" t="s">
+      <c r="F20" s="27" t="s">
         <v>1</v>
       </c>
-      <c r="G20" s="39"/>
-      <c r="H20" s="33" t="s">
+      <c r="G20" s="28"/>
+      <c r="H20" s="40" t="s">
         <v>2</v>
       </c>
-      <c r="I20" s="33"/>
+      <c r="I20" s="40"/>
       <c r="J20" s="8"/>
     </row>
     <row r="21" spans="2:10" x14ac:dyDescent="0.3">
       <c r="B21" s="3"/>
-      <c r="C21" s="36" t="s">
+      <c r="C21" s="26" t="s">
         <v>3</v>
       </c>
-      <c r="D21" s="36"/>
-      <c r="E21" s="36"/>
+      <c r="D21" s="26"/>
+      <c r="E21" s="26"/>
       <c r="F21" s="18"/>
       <c r="G21" s="19"/>
       <c r="H21" s="16"/>
@@ -1099,11 +1095,11 @@
     </row>
     <row r="22" spans="2:10" x14ac:dyDescent="0.3">
       <c r="B22" s="3"/>
-      <c r="C22" s="35" t="s">
+      <c r="C22" s="25" t="s">
         <v>4</v>
       </c>
-      <c r="D22" s="35"/>
-      <c r="E22" s="35"/>
+      <c r="D22" s="25"/>
+      <c r="E22" s="25"/>
       <c r="F22" s="16"/>
       <c r="G22" s="17"/>
       <c r="H22" s="16"/>
@@ -1112,11 +1108,11 @@
     </row>
     <row r="23" spans="2:10" x14ac:dyDescent="0.3">
       <c r="B23" s="3"/>
-      <c r="C23" s="35" t="s">
+      <c r="C23" s="25" t="s">
         <v>5</v>
       </c>
-      <c r="D23" s="35"/>
-      <c r="E23" s="35"/>
+      <c r="D23" s="25"/>
+      <c r="E23" s="25"/>
       <c r="F23" s="16"/>
       <c r="G23" s="17"/>
       <c r="H23" s="16"/>
@@ -1125,11 +1121,11 @@
     </row>
     <row r="24" spans="2:10" x14ac:dyDescent="0.3">
       <c r="B24" s="3"/>
-      <c r="C24" s="29" t="s">
+      <c r="C24" s="36" t="s">
         <v>11</v>
       </c>
-      <c r="D24" s="29"/>
-      <c r="E24" s="29"/>
+      <c r="D24" s="36"/>
+      <c r="E24" s="36"/>
       <c r="F24" s="18"/>
       <c r="G24" s="19"/>
       <c r="H24" s="18"/>
@@ -1137,11 +1133,11 @@
     </row>
     <row r="25" spans="2:10" x14ac:dyDescent="0.3">
       <c r="B25" s="3"/>
-      <c r="C25" s="29" t="s">
+      <c r="C25" s="36" t="s">
         <v>12</v>
       </c>
-      <c r="D25" s="29"/>
-      <c r="E25" s="29"/>
+      <c r="D25" s="36"/>
+      <c r="E25" s="36"/>
       <c r="F25" s="18"/>
       <c r="G25" s="19"/>
       <c r="H25" s="18"/>
@@ -1149,11 +1145,11 @@
     </row>
     <row r="26" spans="2:10" x14ac:dyDescent="0.3">
       <c r="B26" s="3"/>
-      <c r="C26" s="37" t="s">
+      <c r="C26" s="42" t="s">
         <v>6</v>
       </c>
-      <c r="D26" s="37"/>
-      <c r="E26" s="37"/>
+      <c r="D26" s="42"/>
+      <c r="E26" s="42"/>
       <c r="F26" s="16"/>
       <c r="G26" s="17"/>
       <c r="H26" s="16"/>
@@ -1162,10 +1158,10 @@
     </row>
     <row r="27" spans="2:10" x14ac:dyDescent="0.3">
       <c r="B27" s="3"/>
-      <c r="C27" s="34" t="s">
+      <c r="C27" s="41" t="s">
         <v>13</v>
       </c>
-      <c r="D27" s="34"/>
+      <c r="D27" s="41"/>
       <c r="F27" s="18"/>
       <c r="G27" s="19"/>
       <c r="H27" s="18"/>
@@ -1184,10 +1180,10 @@
     </row>
     <row r="29" spans="2:10" x14ac:dyDescent="0.3">
       <c r="B29" s="3"/>
-      <c r="C29" s="35" t="s">
+      <c r="C29" s="25" t="s">
         <v>7</v>
       </c>
-      <c r="D29" s="35"/>
+      <c r="D29" s="25"/>
       <c r="E29" s="10"/>
       <c r="F29" s="16"/>
       <c r="G29" s="17"/>
@@ -1197,10 +1193,10 @@
     </row>
     <row r="30" spans="2:10" x14ac:dyDescent="0.3">
       <c r="B30" s="3"/>
-      <c r="C30" s="36" t="s">
+      <c r="C30" s="26" t="s">
         <v>8</v>
       </c>
-      <c r="D30" s="36"/>
+      <c r="D30" s="26"/>
       <c r="E30" s="10"/>
       <c r="F30" s="20"/>
       <c r="G30" s="21"/>
@@ -1220,61 +1216,56 @@
       <c r="J31" s="4"/>
     </row>
     <row r="32" spans="2:10" ht="31.8" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B32" s="30" t="s">
+      <c r="B32" s="37" t="s">
         <v>9</v>
       </c>
-      <c r="C32" s="31"/>
-      <c r="D32" s="31"/>
-      <c r="E32" s="31"/>
-      <c r="F32" s="31"/>
-      <c r="G32" s="31"/>
-      <c r="H32" s="31"/>
-      <c r="I32" s="31"/>
-      <c r="J32" s="32"/>
+      <c r="C32" s="38"/>
+      <c r="D32" s="38"/>
+      <c r="E32" s="38"/>
+      <c r="F32" s="38"/>
+      <c r="G32" s="38"/>
+      <c r="H32" s="38"/>
+      <c r="I32" s="38"/>
+      <c r="J32" s="39"/>
     </row>
     <row r="36" spans="2:10" ht="39.6" customHeight="1" x14ac:dyDescent="0.3"/>
     <row r="37" spans="2:10" x14ac:dyDescent="0.3">
-      <c r="B37" s="26"/>
-      <c r="C37" s="26"/>
-      <c r="D37" s="26"/>
-      <c r="E37" s="26"/>
-      <c r="F37" s="26"/>
-      <c r="G37" s="26"/>
-      <c r="H37" s="26"/>
-      <c r="I37" s="26"/>
-      <c r="J37" s="26"/>
+      <c r="B37" s="33"/>
+      <c r="C37" s="33"/>
+      <c r="D37" s="33"/>
+      <c r="E37" s="33"/>
+      <c r="F37" s="33"/>
+      <c r="G37" s="33"/>
+      <c r="H37" s="33"/>
+      <c r="I37" s="33"/>
+      <c r="J37" s="33"/>
     </row>
     <row r="38" spans="2:10" x14ac:dyDescent="0.3">
-      <c r="B38" s="27"/>
-      <c r="C38" s="27"/>
-      <c r="D38" s="27"/>
-      <c r="E38" s="27"/>
-      <c r="F38" s="27"/>
-      <c r="G38" s="27"/>
-      <c r="H38" s="27"/>
-      <c r="I38" s="27"/>
-      <c r="J38" s="27"/>
+      <c r="B38" s="34"/>
+      <c r="C38" s="34"/>
+      <c r="D38" s="34"/>
+      <c r="E38" s="34"/>
+      <c r="F38" s="34"/>
+      <c r="G38" s="34"/>
+      <c r="H38" s="34"/>
+      <c r="I38" s="34"/>
+      <c r="J38" s="34"/>
     </row>
     <row r="39" spans="2:10" x14ac:dyDescent="0.3">
-      <c r="B39" s="27"/>
-      <c r="C39" s="27"/>
-      <c r="D39" s="27"/>
-      <c r="E39" s="27"/>
-      <c r="F39" s="27"/>
-      <c r="G39" s="27"/>
-      <c r="H39" s="27"/>
-      <c r="I39" s="27"/>
-      <c r="J39" s="27"/>
+      <c r="B39" s="34"/>
+      <c r="C39" s="34"/>
+      <c r="D39" s="34"/>
+      <c r="E39" s="34"/>
+      <c r="F39" s="34"/>
+      <c r="G39" s="34"/>
+      <c r="H39" s="34"/>
+      <c r="I39" s="34"/>
+      <c r="J39" s="34"/>
     </row>
     <row r="44" spans="2:10" ht="58.2" customHeight="1" x14ac:dyDescent="0.3"/>
     <row r="46" spans="2:10" ht="59.4" customHeight="1" x14ac:dyDescent="0.3"/>
   </sheetData>
   <mergeCells count="20">
-    <mergeCell ref="C22:E22"/>
-    <mergeCell ref="C21:E21"/>
-    <mergeCell ref="F20:G20"/>
-    <mergeCell ref="B15:J15"/>
-    <mergeCell ref="B12:E12"/>
     <mergeCell ref="B37:J37"/>
     <mergeCell ref="B38:J38"/>
     <mergeCell ref="B39:J39"/>
@@ -1290,6 +1281,11 @@
     <mergeCell ref="C26:E26"/>
     <mergeCell ref="C24:E24"/>
     <mergeCell ref="C23:E23"/>
+    <mergeCell ref="C22:E22"/>
+    <mergeCell ref="C21:E21"/>
+    <mergeCell ref="F20:G20"/>
+    <mergeCell ref="B15:J15"/>
+    <mergeCell ref="B12:E12"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>

</xml_diff>

<commit_message>
Update binary files for formato templates
</commit_message>
<xml_diff>
--- a/templates/formato.xlsx
+++ b/templates/formato.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/e039d0c270e9facf/Desktop/Developer/UANL---LABORATORIO-DE-ALIMENTOS-MEDICAMENTOS-Y-TOXICOLOGIA/templates/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="104" documentId="8_{47FAC42F-AC07-43D6-8172-01CEADEBF0F6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{C3267699-BD39-4B78-AAA5-A7E550DEE5E0}"/>
+  <xr:revisionPtr revIDLastSave="106" documentId="8_{47FAC42F-AC07-43D6-8172-01CEADEBF0F6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{9D674C6D-B2CB-4497-AEE2-8A4548CC5D69}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{1CB8A4CE-E91B-448F-9BE6-E546BA7C8907}"/>
   </bookViews>
@@ -377,15 +377,33 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="14" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="15" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="16" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -416,28 +434,16 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
   </cellXfs>
@@ -582,10 +588,6 @@
     <xdr:clientData/>
   </xdr:twoCellAnchor>
 </xdr:wsDr>
-</file>
-
-<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
-<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -921,28 +923,28 @@
   </cols>
   <sheetData>
     <row r="4" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A4" s="27"/>
-      <c r="B4" s="27"/>
-      <c r="C4" s="27"/>
-      <c r="D4" s="27"/>
-      <c r="E4" s="27"/>
-      <c r="F4" s="27"/>
-      <c r="G4" s="27"/>
-      <c r="H4" s="27"/>
-      <c r="I4" s="27"/>
-      <c r="J4" s="27"/>
+      <c r="A4" s="31"/>
+      <c r="B4" s="31"/>
+      <c r="C4" s="31"/>
+      <c r="D4" s="31"/>
+      <c r="E4" s="31"/>
+      <c r="F4" s="31"/>
+      <c r="G4" s="31"/>
+      <c r="H4" s="31"/>
+      <c r="I4" s="31"/>
+      <c r="J4" s="31"/>
     </row>
     <row r="5" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A5" s="27"/>
-      <c r="B5" s="27"/>
-      <c r="C5" s="27"/>
-      <c r="D5" s="27"/>
-      <c r="E5" s="27"/>
-      <c r="F5" s="27"/>
-      <c r="G5" s="27"/>
-      <c r="H5" s="27"/>
-      <c r="I5" s="27"/>
-      <c r="J5" s="27"/>
+      <c r="A5" s="31"/>
+      <c r="B5" s="31"/>
+      <c r="C5" s="31"/>
+      <c r="D5" s="31"/>
+      <c r="E5" s="31"/>
+      <c r="F5" s="31"/>
+      <c r="G5" s="31"/>
+      <c r="H5" s="31"/>
+      <c r="I5" s="31"/>
+      <c r="J5" s="31"/>
     </row>
     <row r="6" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A6" s="1"/>
@@ -969,7 +971,7 @@
       <c r="J7" s="1"/>
     </row>
     <row r="8" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="B8" s="22" t="s">
+      <c r="B8" s="19" t="s">
         <v>18</v>
       </c>
       <c r="C8" s="13"/>
@@ -982,25 +984,25 @@
       <c r="J8" s="2"/>
     </row>
     <row r="10" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="B10" s="28" t="s">
+      <c r="B10" s="32" t="s">
         <v>0</v>
       </c>
-      <c r="C10" s="28"/>
-      <c r="D10" s="28"/>
-      <c r="E10" s="28"/>
-      <c r="F10" s="28"/>
-      <c r="G10" s="28"/>
-      <c r="H10" s="28"/>
-      <c r="I10" s="28"/>
-      <c r="J10" s="28"/>
+      <c r="C10" s="32"/>
+      <c r="D10" s="32"/>
+      <c r="E10" s="32"/>
+      <c r="F10" s="32"/>
+      <c r="G10" s="32"/>
+      <c r="H10" s="32"/>
+      <c r="I10" s="32"/>
+      <c r="J10" s="32"/>
     </row>
     <row r="12" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="B12" s="42" t="s">
+      <c r="B12" s="28" t="s">
         <v>17</v>
       </c>
-      <c r="C12" s="42"/>
-      <c r="D12" s="42"/>
-      <c r="E12" s="42"/>
+      <c r="C12" s="28"/>
+      <c r="D12" s="28"/>
+      <c r="E12" s="28"/>
     </row>
     <row r="13" spans="1:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
     <row r="14" spans="1:10" x14ac:dyDescent="0.25">
@@ -1015,17 +1017,17 @@
       <c r="J14" s="7"/>
     </row>
     <row r="15" spans="1:10" ht="21" x14ac:dyDescent="0.35">
-      <c r="B15" s="39" t="s">
+      <c r="B15" s="25" t="s">
         <v>9</v>
       </c>
-      <c r="C15" s="40"/>
-      <c r="D15" s="40"/>
-      <c r="E15" s="40"/>
-      <c r="F15" s="40"/>
-      <c r="G15" s="40"/>
-      <c r="H15" s="40"/>
-      <c r="I15" s="40"/>
-      <c r="J15" s="41"/>
+      <c r="C15" s="26"/>
+      <c r="D15" s="26"/>
+      <c r="E15" s="26"/>
+      <c r="F15" s="26"/>
+      <c r="G15" s="26"/>
+      <c r="H15" s="26"/>
+      <c r="I15" s="26"/>
+      <c r="J15" s="27"/>
     </row>
     <row r="16" spans="1:10" x14ac:dyDescent="0.25">
       <c r="B16" s="3"/>
@@ -1033,10 +1035,10 @@
     </row>
     <row r="17" spans="2:10" x14ac:dyDescent="0.25">
       <c r="B17" s="3"/>
-      <c r="C17" s="23" t="s">
+      <c r="C17" s="20" t="s">
         <v>14</v>
       </c>
-      <c r="D17" s="23"/>
+      <c r="D17" s="20"/>
       <c r="E17" s="10"/>
       <c r="F17" s="12"/>
       <c r="G17" s="10"/>
@@ -1046,10 +1048,10 @@
     </row>
     <row r="18" spans="2:10" x14ac:dyDescent="0.25">
       <c r="B18" s="3"/>
-      <c r="C18" s="23" t="s">
+      <c r="C18" s="20" t="s">
         <v>15</v>
       </c>
-      <c r="D18" s="23"/>
+      <c r="D18" s="20"/>
       <c r="E18" s="12"/>
       <c r="G18" s="12"/>
       <c r="H18" s="11"/>
@@ -1058,11 +1060,11 @@
     </row>
     <row r="19" spans="2:10" x14ac:dyDescent="0.25">
       <c r="B19" s="3"/>
-      <c r="C19" s="24" t="s">
+      <c r="C19" s="21" t="s">
         <v>16</v>
       </c>
-      <c r="D19" s="24"/>
-      <c r="E19" s="24"/>
+      <c r="D19" s="21"/>
+      <c r="E19" s="21"/>
       <c r="F19" s="15"/>
       <c r="G19" s="15"/>
       <c r="H19" s="14"/>
@@ -1074,101 +1076,101 @@
       <c r="C20" s="10"/>
       <c r="D20" s="10"/>
       <c r="E20" s="10"/>
-      <c r="F20" s="37" t="s">
+      <c r="F20" s="23" t="s">
         <v>19</v>
       </c>
-      <c r="G20" s="38"/>
-      <c r="H20" s="32" t="s">
+      <c r="G20" s="24"/>
+      <c r="H20" s="36" t="s">
         <v>1</v>
       </c>
-      <c r="I20" s="32"/>
+      <c r="I20" s="36"/>
       <c r="J20" s="8"/>
     </row>
     <row r="21" spans="2:10" x14ac:dyDescent="0.25">
       <c r="B21" s="3"/>
-      <c r="C21" s="35" t="s">
+      <c r="C21" s="22" t="s">
         <v>2</v>
       </c>
-      <c r="D21" s="35"/>
-      <c r="E21" s="35"/>
-      <c r="F21" s="18"/>
-      <c r="G21" s="19"/>
-      <c r="H21" s="16"/>
+      <c r="D21" s="22"/>
+      <c r="E21" s="22"/>
+      <c r="F21" s="40"/>
+      <c r="G21" s="17"/>
+      <c r="H21" s="41"/>
       <c r="I21" s="10"/>
       <c r="J21" s="9"/>
     </row>
     <row r="22" spans="2:10" x14ac:dyDescent="0.25">
       <c r="B22" s="3"/>
-      <c r="C22" s="34" t="s">
+      <c r="C22" s="38" t="s">
         <v>3</v>
       </c>
-      <c r="D22" s="34"/>
-      <c r="E22" s="34"/>
-      <c r="F22" s="16"/>
-      <c r="G22" s="17"/>
-      <c r="H22" s="16"/>
+      <c r="D22" s="38"/>
+      <c r="E22" s="38"/>
+      <c r="F22" s="41"/>
+      <c r="G22" s="16"/>
+      <c r="H22" s="41"/>
       <c r="I22" s="10"/>
       <c r="J22" s="8"/>
     </row>
     <row r="23" spans="2:10" x14ac:dyDescent="0.25">
       <c r="B23" s="3"/>
-      <c r="C23" s="34" t="s">
+      <c r="C23" s="38" t="s">
         <v>4</v>
       </c>
-      <c r="D23" s="34"/>
-      <c r="E23" s="34"/>
-      <c r="F23" s="16"/>
-      <c r="G23" s="17"/>
-      <c r="H23" s="16"/>
+      <c r="D23" s="38"/>
+      <c r="E23" s="38"/>
+      <c r="F23" s="41"/>
+      <c r="G23" s="16"/>
+      <c r="H23" s="41"/>
       <c r="I23" s="10"/>
       <c r="J23" s="8"/>
     </row>
     <row r="24" spans="2:10" x14ac:dyDescent="0.25">
       <c r="B24" s="3"/>
-      <c r="C24" s="28" t="s">
+      <c r="C24" s="32" t="s">
         <v>10</v>
       </c>
-      <c r="D24" s="28"/>
-      <c r="E24" s="28"/>
-      <c r="F24" s="18"/>
-      <c r="G24" s="19"/>
-      <c r="H24" s="18"/>
+      <c r="D24" s="32"/>
+      <c r="E24" s="32"/>
+      <c r="F24" s="40"/>
+      <c r="G24" s="17"/>
+      <c r="H24" s="40"/>
       <c r="J24" s="8"/>
     </row>
     <row r="25" spans="2:10" x14ac:dyDescent="0.25">
       <c r="B25" s="3"/>
-      <c r="C25" s="28" t="s">
+      <c r="C25" s="32" t="s">
         <v>11</v>
       </c>
-      <c r="D25" s="28"/>
-      <c r="E25" s="28"/>
-      <c r="F25" s="18"/>
-      <c r="G25" s="19"/>
-      <c r="H25" s="18"/>
+      <c r="D25" s="32"/>
+      <c r="E25" s="32"/>
+      <c r="F25" s="40"/>
+      <c r="G25" s="17"/>
+      <c r="H25" s="40"/>
       <c r="J25" s="8"/>
     </row>
     <row r="26" spans="2:10" x14ac:dyDescent="0.25">
       <c r="B26" s="3"/>
-      <c r="C26" s="36" t="s">
+      <c r="C26" s="39" t="s">
         <v>5</v>
       </c>
-      <c r="D26" s="36"/>
-      <c r="E26" s="36"/>
-      <c r="F26" s="16"/>
-      <c r="G26" s="17"/>
-      <c r="H26" s="16"/>
+      <c r="D26" s="39"/>
+      <c r="E26" s="39"/>
+      <c r="F26" s="41"/>
+      <c r="G26" s="16"/>
+      <c r="H26" s="41"/>
       <c r="I26" s="10"/>
       <c r="J26" s="8"/>
     </row>
     <row r="27" spans="2:10" x14ac:dyDescent="0.25">
       <c r="B27" s="3"/>
-      <c r="C27" s="33" t="s">
+      <c r="C27" s="37" t="s">
         <v>12</v>
       </c>
-      <c r="D27" s="33"/>
-      <c r="F27" s="18"/>
-      <c r="G27" s="19"/>
-      <c r="H27" s="18"/>
+      <c r="D27" s="37"/>
+      <c r="F27" s="40"/>
+      <c r="G27" s="17"/>
+      <c r="H27" s="40"/>
       <c r="J27" s="8"/>
     </row>
     <row r="28" spans="2:10" x14ac:dyDescent="0.25">
@@ -1177,34 +1179,34 @@
         <v>13</v>
       </c>
       <c r="D28" s="13"/>
-      <c r="F28" s="18"/>
-      <c r="G28" s="19"/>
-      <c r="H28" s="18"/>
+      <c r="F28" s="40"/>
+      <c r="G28" s="17"/>
+      <c r="H28" s="40"/>
       <c r="J28" s="8"/>
     </row>
     <row r="29" spans="2:10" x14ac:dyDescent="0.25">
       <c r="B29" s="3"/>
-      <c r="C29" s="34" t="s">
+      <c r="C29" s="38" t="s">
         <v>6</v>
       </c>
-      <c r="D29" s="34"/>
+      <c r="D29" s="38"/>
       <c r="E29" s="10"/>
-      <c r="F29" s="16"/>
-      <c r="G29" s="17"/>
-      <c r="H29" s="16"/>
+      <c r="F29" s="41"/>
+      <c r="G29" s="16"/>
+      <c r="H29" s="41"/>
       <c r="I29" s="10"/>
       <c r="J29" s="8"/>
     </row>
     <row r="30" spans="2:10" x14ac:dyDescent="0.25">
       <c r="B30" s="3"/>
-      <c r="C30" s="35" t="s">
+      <c r="C30" s="22" t="s">
         <v>7</v>
       </c>
-      <c r="D30" s="35"/>
+      <c r="D30" s="22"/>
       <c r="E30" s="10"/>
-      <c r="F30" s="20"/>
-      <c r="G30" s="21"/>
-      <c r="H30" s="20"/>
+      <c r="F30" s="42"/>
+      <c r="G30" s="18"/>
+      <c r="H30" s="42"/>
       <c r="I30" s="12"/>
       <c r="J30" s="8"/>
     </row>
@@ -1220,61 +1222,56 @@
       <c r="J31" s="4"/>
     </row>
     <row r="32" spans="2:10" ht="31.9" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B32" s="29" t="s">
+      <c r="B32" s="33" t="s">
         <v>8</v>
       </c>
-      <c r="C32" s="30"/>
-      <c r="D32" s="30"/>
-      <c r="E32" s="30"/>
-      <c r="F32" s="30"/>
-      <c r="G32" s="30"/>
-      <c r="H32" s="30"/>
-      <c r="I32" s="30"/>
-      <c r="J32" s="31"/>
+      <c r="C32" s="34"/>
+      <c r="D32" s="34"/>
+      <c r="E32" s="34"/>
+      <c r="F32" s="34"/>
+      <c r="G32" s="34"/>
+      <c r="H32" s="34"/>
+      <c r="I32" s="34"/>
+      <c r="J32" s="35"/>
     </row>
     <row r="36" spans="2:10" ht="39.6" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="37" spans="2:10" x14ac:dyDescent="0.25">
-      <c r="B37" s="25"/>
-      <c r="C37" s="25"/>
-      <c r="D37" s="25"/>
-      <c r="E37" s="25"/>
-      <c r="F37" s="25"/>
-      <c r="G37" s="25"/>
-      <c r="H37" s="25"/>
-      <c r="I37" s="25"/>
-      <c r="J37" s="25"/>
+      <c r="B37" s="29"/>
+      <c r="C37" s="29"/>
+      <c r="D37" s="29"/>
+      <c r="E37" s="29"/>
+      <c r="F37" s="29"/>
+      <c r="G37" s="29"/>
+      <c r="H37" s="29"/>
+      <c r="I37" s="29"/>
+      <c r="J37" s="29"/>
     </row>
     <row r="38" spans="2:10" x14ac:dyDescent="0.25">
-      <c r="B38" s="26"/>
-      <c r="C38" s="26"/>
-      <c r="D38" s="26"/>
-      <c r="E38" s="26"/>
-      <c r="F38" s="26"/>
-      <c r="G38" s="26"/>
-      <c r="H38" s="26"/>
-      <c r="I38" s="26"/>
-      <c r="J38" s="26"/>
+      <c r="B38" s="30"/>
+      <c r="C38" s="30"/>
+      <c r="D38" s="30"/>
+      <c r="E38" s="30"/>
+      <c r="F38" s="30"/>
+      <c r="G38" s="30"/>
+      <c r="H38" s="30"/>
+      <c r="I38" s="30"/>
+      <c r="J38" s="30"/>
     </row>
     <row r="39" spans="2:10" x14ac:dyDescent="0.25">
-      <c r="B39" s="26"/>
-      <c r="C39" s="26"/>
-      <c r="D39" s="26"/>
-      <c r="E39" s="26"/>
-      <c r="F39" s="26"/>
-      <c r="G39" s="26"/>
-      <c r="H39" s="26"/>
-      <c r="I39" s="26"/>
-      <c r="J39" s="26"/>
+      <c r="B39" s="30"/>
+      <c r="C39" s="30"/>
+      <c r="D39" s="30"/>
+      <c r="E39" s="30"/>
+      <c r="F39" s="30"/>
+      <c r="G39" s="30"/>
+      <c r="H39" s="30"/>
+      <c r="I39" s="30"/>
+      <c r="J39" s="30"/>
     </row>
     <row r="44" spans="2:10" ht="58.15" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="46" spans="2:10" ht="59.45" customHeight="1" x14ac:dyDescent="0.25"/>
   </sheetData>
   <mergeCells count="20">
-    <mergeCell ref="C21:E21"/>
-    <mergeCell ref="F20:G20"/>
-    <mergeCell ref="B15:J15"/>
-    <mergeCell ref="B12:E12"/>
-    <mergeCell ref="B37:J37"/>
     <mergeCell ref="B38:J38"/>
     <mergeCell ref="B39:J39"/>
     <mergeCell ref="A4:J4"/>
@@ -1290,6 +1287,11 @@
     <mergeCell ref="C24:E24"/>
     <mergeCell ref="C23:E23"/>
     <mergeCell ref="C22:E22"/>
+    <mergeCell ref="C21:E21"/>
+    <mergeCell ref="F20:G20"/>
+    <mergeCell ref="B15:J15"/>
+    <mergeCell ref="B12:E12"/>
+    <mergeCell ref="B37:J37"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>

</xml_diff>

<commit_message>
Add left alignment function for merged cells in NutrimentalExporter
</commit_message>
<xml_diff>
--- a/templates/formato.xlsx
+++ b/templates/formato.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29127"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29231"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/e039d0c270e9facf/Desktop/Developer/UANL---LABORATORIO-DE-ALIMENTOS-MEDICAMENTOS-Y-TOXICOLOGIA/templates/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="106" documentId="8_{47FAC42F-AC07-43D6-8172-01CEADEBF0F6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{9D674C6D-B2CB-4497-AEE2-8A4548CC5D69}"/>
+  <xr:revisionPtr revIDLastSave="109" documentId="8_{47FAC42F-AC07-43D6-8172-01CEADEBF0F6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{5125B583-54AC-4CFA-9CB9-E97CA7F09106}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{1CB8A4CE-E91B-448F-9BE6-E546BA7C8907}"/>
   </bookViews>
@@ -95,7 +95,7 @@
     <t xml:space="preserve">MUESTRA: </t>
   </si>
   <si>
-    <t>Por 100 g</t>
+    <t>Por 100</t>
   </si>
 </sst>
 </file>
@@ -383,14 +383,53 @@
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -406,45 +445,6 @@
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -588,6 +588,10 @@
     <xdr:clientData/>
   </xdr:twoCellAnchor>
 </xdr:wsDr>
+</file>
+
+<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
+<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -923,28 +927,28 @@
   </cols>
   <sheetData>
     <row r="4" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A4" s="31"/>
-      <c r="B4" s="31"/>
-      <c r="C4" s="31"/>
-      <c r="D4" s="31"/>
-      <c r="E4" s="31"/>
-      <c r="F4" s="31"/>
-      <c r="G4" s="31"/>
-      <c r="H4" s="31"/>
-      <c r="I4" s="31"/>
-      <c r="J4" s="31"/>
+      <c r="A4" s="28"/>
+      <c r="B4" s="28"/>
+      <c r="C4" s="28"/>
+      <c r="D4" s="28"/>
+      <c r="E4" s="28"/>
+      <c r="F4" s="28"/>
+      <c r="G4" s="28"/>
+      <c r="H4" s="28"/>
+      <c r="I4" s="28"/>
+      <c r="J4" s="28"/>
     </row>
     <row r="5" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A5" s="31"/>
-      <c r="B5" s="31"/>
-      <c r="C5" s="31"/>
-      <c r="D5" s="31"/>
-      <c r="E5" s="31"/>
-      <c r="F5" s="31"/>
-      <c r="G5" s="31"/>
-      <c r="H5" s="31"/>
-      <c r="I5" s="31"/>
-      <c r="J5" s="31"/>
+      <c r="A5" s="28"/>
+      <c r="B5" s="28"/>
+      <c r="C5" s="28"/>
+      <c r="D5" s="28"/>
+      <c r="E5" s="28"/>
+      <c r="F5" s="28"/>
+      <c r="G5" s="28"/>
+      <c r="H5" s="28"/>
+      <c r="I5" s="28"/>
+      <c r="J5" s="28"/>
     </row>
     <row r="6" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A6" s="1"/>
@@ -984,25 +988,25 @@
       <c r="J8" s="2"/>
     </row>
     <row r="10" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="B10" s="32" t="s">
+      <c r="B10" s="29" t="s">
         <v>0</v>
       </c>
-      <c r="C10" s="32"/>
-      <c r="D10" s="32"/>
-      <c r="E10" s="32"/>
-      <c r="F10" s="32"/>
-      <c r="G10" s="32"/>
-      <c r="H10" s="32"/>
-      <c r="I10" s="32"/>
-      <c r="J10" s="32"/>
+      <c r="C10" s="29"/>
+      <c r="D10" s="29"/>
+      <c r="E10" s="29"/>
+      <c r="F10" s="29"/>
+      <c r="G10" s="29"/>
+      <c r="H10" s="29"/>
+      <c r="I10" s="29"/>
+      <c r="J10" s="29"/>
     </row>
     <row r="12" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="B12" s="28" t="s">
+      <c r="B12" s="41" t="s">
         <v>17</v>
       </c>
-      <c r="C12" s="28"/>
-      <c r="D12" s="28"/>
-      <c r="E12" s="28"/>
+      <c r="C12" s="41"/>
+      <c r="D12" s="41"/>
+      <c r="E12" s="41"/>
     </row>
     <row r="13" spans="1:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
     <row r="14" spans="1:10" x14ac:dyDescent="0.25">
@@ -1017,17 +1021,17 @@
       <c r="J14" s="7"/>
     </row>
     <row r="15" spans="1:10" ht="21" x14ac:dyDescent="0.35">
-      <c r="B15" s="25" t="s">
+      <c r="B15" s="38" t="s">
         <v>9</v>
       </c>
-      <c r="C15" s="26"/>
-      <c r="D15" s="26"/>
-      <c r="E15" s="26"/>
-      <c r="F15" s="26"/>
-      <c r="G15" s="26"/>
-      <c r="H15" s="26"/>
-      <c r="I15" s="26"/>
-      <c r="J15" s="27"/>
+      <c r="C15" s="39"/>
+      <c r="D15" s="39"/>
+      <c r="E15" s="39"/>
+      <c r="F15" s="39"/>
+      <c r="G15" s="39"/>
+      <c r="H15" s="39"/>
+      <c r="I15" s="39"/>
+      <c r="J15" s="40"/>
     </row>
     <row r="16" spans="1:10" x14ac:dyDescent="0.25">
       <c r="B16" s="3"/>
@@ -1076,101 +1080,101 @@
       <c r="C20" s="10"/>
       <c r="D20" s="10"/>
       <c r="E20" s="10"/>
-      <c r="F20" s="23" t="s">
+      <c r="F20" s="22" t="s">
         <v>19</v>
       </c>
-      <c r="G20" s="24"/>
-      <c r="H20" s="36" t="s">
+      <c r="G20" s="23"/>
+      <c r="H20" s="33" t="s">
         <v>1</v>
       </c>
-      <c r="I20" s="36"/>
+      <c r="I20" s="33"/>
       <c r="J20" s="8"/>
     </row>
     <row r="21" spans="2:10" x14ac:dyDescent="0.25">
       <c r="B21" s="3"/>
-      <c r="C21" s="22" t="s">
+      <c r="C21" s="36" t="s">
         <v>2</v>
       </c>
-      <c r="D21" s="22"/>
-      <c r="E21" s="22"/>
-      <c r="F21" s="40"/>
+      <c r="D21" s="36"/>
+      <c r="E21" s="36"/>
+      <c r="F21" s="24"/>
       <c r="G21" s="17"/>
-      <c r="H21" s="41"/>
+      <c r="H21" s="25"/>
       <c r="I21" s="10"/>
       <c r="J21" s="9"/>
     </row>
     <row r="22" spans="2:10" x14ac:dyDescent="0.25">
       <c r="B22" s="3"/>
-      <c r="C22" s="38" t="s">
+      <c r="C22" s="35" t="s">
         <v>3</v>
       </c>
-      <c r="D22" s="38"/>
-      <c r="E22" s="38"/>
-      <c r="F22" s="41"/>
+      <c r="D22" s="35"/>
+      <c r="E22" s="35"/>
+      <c r="F22" s="25"/>
       <c r="G22" s="16"/>
-      <c r="H22" s="41"/>
+      <c r="H22" s="25"/>
       <c r="I22" s="10"/>
       <c r="J22" s="8"/>
     </row>
     <row r="23" spans="2:10" x14ac:dyDescent="0.25">
       <c r="B23" s="3"/>
-      <c r="C23" s="38" t="s">
+      <c r="C23" s="35" t="s">
         <v>4</v>
       </c>
-      <c r="D23" s="38"/>
-      <c r="E23" s="38"/>
-      <c r="F23" s="41"/>
+      <c r="D23" s="35"/>
+      <c r="E23" s="35"/>
+      <c r="F23" s="25"/>
       <c r="G23" s="16"/>
-      <c r="H23" s="41"/>
+      <c r="H23" s="25"/>
       <c r="I23" s="10"/>
       <c r="J23" s="8"/>
     </row>
     <row r="24" spans="2:10" x14ac:dyDescent="0.25">
       <c r="B24" s="3"/>
-      <c r="C24" s="32" t="s">
+      <c r="C24" s="29" t="s">
         <v>10</v>
       </c>
-      <c r="D24" s="32"/>
-      <c r="E24" s="32"/>
-      <c r="F24" s="40"/>
+      <c r="D24" s="29"/>
+      <c r="E24" s="29"/>
+      <c r="F24" s="24"/>
       <c r="G24" s="17"/>
-      <c r="H24" s="40"/>
+      <c r="H24" s="24"/>
       <c r="J24" s="8"/>
     </row>
     <row r="25" spans="2:10" x14ac:dyDescent="0.25">
       <c r="B25" s="3"/>
-      <c r="C25" s="32" t="s">
+      <c r="C25" s="29" t="s">
         <v>11</v>
       </c>
-      <c r="D25" s="32"/>
-      <c r="E25" s="32"/>
-      <c r="F25" s="40"/>
+      <c r="D25" s="29"/>
+      <c r="E25" s="29"/>
+      <c r="F25" s="24"/>
       <c r="G25" s="17"/>
-      <c r="H25" s="40"/>
+      <c r="H25" s="24"/>
       <c r="J25" s="8"/>
     </row>
     <row r="26" spans="2:10" x14ac:dyDescent="0.25">
       <c r="B26" s="3"/>
-      <c r="C26" s="39" t="s">
+      <c r="C26" s="37" t="s">
         <v>5</v>
       </c>
-      <c r="D26" s="39"/>
-      <c r="E26" s="39"/>
-      <c r="F26" s="41"/>
+      <c r="D26" s="37"/>
+      <c r="E26" s="37"/>
+      <c r="F26" s="25"/>
       <c r="G26" s="16"/>
-      <c r="H26" s="41"/>
+      <c r="H26" s="25"/>
       <c r="I26" s="10"/>
       <c r="J26" s="8"/>
     </row>
     <row r="27" spans="2:10" x14ac:dyDescent="0.25">
       <c r="B27" s="3"/>
-      <c r="C27" s="37" t="s">
+      <c r="C27" s="34" t="s">
         <v>12</v>
       </c>
-      <c r="D27" s="37"/>
-      <c r="F27" s="40"/>
+      <c r="D27" s="34"/>
+      <c r="F27" s="24"/>
       <c r="G27" s="17"/>
-      <c r="H27" s="40"/>
+      <c r="H27" s="24"/>
       <c r="J27" s="8"/>
     </row>
     <row r="28" spans="2:10" x14ac:dyDescent="0.25">
@@ -1179,34 +1183,34 @@
         <v>13</v>
       </c>
       <c r="D28" s="13"/>
-      <c r="F28" s="40"/>
+      <c r="F28" s="24"/>
       <c r="G28" s="17"/>
-      <c r="H28" s="40"/>
+      <c r="H28" s="24"/>
       <c r="J28" s="8"/>
     </row>
     <row r="29" spans="2:10" x14ac:dyDescent="0.25">
       <c r="B29" s="3"/>
-      <c r="C29" s="38" t="s">
+      <c r="C29" s="35" t="s">
         <v>6</v>
       </c>
-      <c r="D29" s="38"/>
+      <c r="D29" s="35"/>
       <c r="E29" s="10"/>
-      <c r="F29" s="41"/>
+      <c r="F29" s="25"/>
       <c r="G29" s="16"/>
-      <c r="H29" s="41"/>
+      <c r="H29" s="25"/>
       <c r="I29" s="10"/>
       <c r="J29" s="8"/>
     </row>
     <row r="30" spans="2:10" x14ac:dyDescent="0.25">
       <c r="B30" s="3"/>
-      <c r="C30" s="22" t="s">
+      <c r="C30" s="36" t="s">
         <v>7</v>
       </c>
-      <c r="D30" s="22"/>
+      <c r="D30" s="36"/>
       <c r="E30" s="10"/>
-      <c r="F30" s="42"/>
+      <c r="F30" s="26"/>
       <c r="G30" s="18"/>
-      <c r="H30" s="42"/>
+      <c r="H30" s="26"/>
       <c r="I30" s="12"/>
       <c r="J30" s="8"/>
     </row>
@@ -1222,56 +1226,59 @@
       <c r="J31" s="4"/>
     </row>
     <row r="32" spans="2:10" ht="31.9" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B32" s="33" t="s">
+      <c r="B32" s="30" t="s">
         <v>8</v>
       </c>
-      <c r="C32" s="34"/>
-      <c r="D32" s="34"/>
-      <c r="E32" s="34"/>
-      <c r="F32" s="34"/>
-      <c r="G32" s="34"/>
-      <c r="H32" s="34"/>
-      <c r="I32" s="34"/>
-      <c r="J32" s="35"/>
+      <c r="C32" s="31"/>
+      <c r="D32" s="31"/>
+      <c r="E32" s="31"/>
+      <c r="F32" s="31"/>
+      <c r="G32" s="31"/>
+      <c r="H32" s="31"/>
+      <c r="I32" s="31"/>
+      <c r="J32" s="32"/>
     </row>
     <row r="36" spans="2:10" ht="39.6" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="37" spans="2:10" x14ac:dyDescent="0.25">
-      <c r="B37" s="29"/>
-      <c r="C37" s="29"/>
-      <c r="D37" s="29"/>
-      <c r="E37" s="29"/>
-      <c r="F37" s="29"/>
-      <c r="G37" s="29"/>
-      <c r="H37" s="29"/>
-      <c r="I37" s="29"/>
-      <c r="J37" s="29"/>
+      <c r="B37" s="42"/>
+      <c r="C37" s="42"/>
+      <c r="D37" s="42"/>
+      <c r="E37" s="42"/>
+      <c r="F37" s="42"/>
+      <c r="G37" s="42"/>
+      <c r="H37" s="42"/>
+      <c r="I37" s="42"/>
+      <c r="J37" s="42"/>
     </row>
     <row r="38" spans="2:10" x14ac:dyDescent="0.25">
-      <c r="B38" s="30"/>
-      <c r="C38" s="30"/>
-      <c r="D38" s="30"/>
-      <c r="E38" s="30"/>
-      <c r="F38" s="30"/>
-      <c r="G38" s="30"/>
-      <c r="H38" s="30"/>
-      <c r="I38" s="30"/>
-      <c r="J38" s="30"/>
+      <c r="B38" s="27"/>
+      <c r="C38" s="27"/>
+      <c r="D38" s="27"/>
+      <c r="E38" s="27"/>
+      <c r="F38" s="27"/>
+      <c r="G38" s="27"/>
+      <c r="H38" s="27"/>
+      <c r="I38" s="27"/>
+      <c r="J38" s="27"/>
     </row>
     <row r="39" spans="2:10" x14ac:dyDescent="0.25">
-      <c r="B39" s="30"/>
-      <c r="C39" s="30"/>
-      <c r="D39" s="30"/>
-      <c r="E39" s="30"/>
-      <c r="F39" s="30"/>
-      <c r="G39" s="30"/>
-      <c r="H39" s="30"/>
-      <c r="I39" s="30"/>
-      <c r="J39" s="30"/>
+      <c r="B39" s="27"/>
+      <c r="C39" s="27"/>
+      <c r="D39" s="27"/>
+      <c r="E39" s="27"/>
+      <c r="F39" s="27"/>
+      <c r="G39" s="27"/>
+      <c r="H39" s="27"/>
+      <c r="I39" s="27"/>
+      <c r="J39" s="27"/>
     </row>
     <row r="44" spans="2:10" ht="58.15" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="46" spans="2:10" ht="59.45" customHeight="1" x14ac:dyDescent="0.25"/>
   </sheetData>
-  <mergeCells count="20">
+  <mergeCells count="19">
+    <mergeCell ref="B15:J15"/>
+    <mergeCell ref="B12:E12"/>
+    <mergeCell ref="B37:J37"/>
     <mergeCell ref="B38:J38"/>
     <mergeCell ref="B39:J39"/>
     <mergeCell ref="A4:J4"/>
@@ -1288,10 +1295,6 @@
     <mergeCell ref="C23:E23"/>
     <mergeCell ref="C22:E22"/>
     <mergeCell ref="C21:E21"/>
-    <mergeCell ref="F20:G20"/>
-    <mergeCell ref="B15:J15"/>
-    <mergeCell ref="B12:E12"/>
-    <mergeCell ref="B37:J37"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>

</xml_diff>

<commit_message>
Align cell contents in NutrimentalExporter and remove unused files
</commit_message>
<xml_diff>
--- a/templates/formato.xlsx
+++ b/templates/formato.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/e039d0c270e9facf/Desktop/Developer/UANL---LABORATORIO-DE-ALIMENTOS-MEDICAMENTOS-Y-TOXICOLOGIA/templates/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="109" documentId="8_{47FAC42F-AC07-43D6-8172-01CEADEBF0F6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{5125B583-54AC-4CFA-9CB9-E97CA7F09106}"/>
+  <xr:revisionPtr revIDLastSave="110" documentId="8_{47FAC42F-AC07-43D6-8172-01CEADEBF0F6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{CF9D600E-358B-48D0-B18F-498332E19149}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{1CB8A4CE-E91B-448F-9BE6-E546BA7C8907}"/>
+    <workbookView xWindow="-23148" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{1CB8A4CE-E91B-448F-9BE6-E546BA7C8907}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -350,7 +350,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="43">
+  <cellXfs count="44">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="right"/>
@@ -398,6 +398,21 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -431,19 +446,7 @@
     <xf numFmtId="0" fontId="6" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="13" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
   </cellXfs>
@@ -927,28 +930,28 @@
   </cols>
   <sheetData>
     <row r="4" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A4" s="28"/>
-      <c r="B4" s="28"/>
-      <c r="C4" s="28"/>
-      <c r="D4" s="28"/>
-      <c r="E4" s="28"/>
-      <c r="F4" s="28"/>
-      <c r="G4" s="28"/>
-      <c r="H4" s="28"/>
-      <c r="I4" s="28"/>
-      <c r="J4" s="28"/>
+      <c r="A4" s="33"/>
+      <c r="B4" s="33"/>
+      <c r="C4" s="33"/>
+      <c r="D4" s="33"/>
+      <c r="E4" s="33"/>
+      <c r="F4" s="33"/>
+      <c r="G4" s="33"/>
+      <c r="H4" s="33"/>
+      <c r="I4" s="33"/>
+      <c r="J4" s="33"/>
     </row>
     <row r="5" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A5" s="28"/>
-      <c r="B5" s="28"/>
-      <c r="C5" s="28"/>
-      <c r="D5" s="28"/>
-      <c r="E5" s="28"/>
-      <c r="F5" s="28"/>
-      <c r="G5" s="28"/>
-      <c r="H5" s="28"/>
-      <c r="I5" s="28"/>
-      <c r="J5" s="28"/>
+      <c r="A5" s="33"/>
+      <c r="B5" s="33"/>
+      <c r="C5" s="33"/>
+      <c r="D5" s="33"/>
+      <c r="E5" s="33"/>
+      <c r="F5" s="33"/>
+      <c r="G5" s="33"/>
+      <c r="H5" s="33"/>
+      <c r="I5" s="33"/>
+      <c r="J5" s="33"/>
     </row>
     <row r="6" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A6" s="1"/>
@@ -988,25 +991,25 @@
       <c r="J8" s="2"/>
     </row>
     <row r="10" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="B10" s="29" t="s">
+      <c r="B10" s="34" t="s">
         <v>0</v>
       </c>
-      <c r="C10" s="29"/>
-      <c r="D10" s="29"/>
-      <c r="E10" s="29"/>
-      <c r="F10" s="29"/>
-      <c r="G10" s="29"/>
-      <c r="H10" s="29"/>
-      <c r="I10" s="29"/>
-      <c r="J10" s="29"/>
+      <c r="C10" s="34"/>
+      <c r="D10" s="34"/>
+      <c r="E10" s="34"/>
+      <c r="F10" s="34"/>
+      <c r="G10" s="34"/>
+      <c r="H10" s="34"/>
+      <c r="I10" s="34"/>
+      <c r="J10" s="34"/>
     </row>
     <row r="12" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="B12" s="41" t="s">
+      <c r="B12" s="30" t="s">
         <v>17</v>
       </c>
-      <c r="C12" s="41"/>
-      <c r="D12" s="41"/>
-      <c r="E12" s="41"/>
+      <c r="C12" s="30"/>
+      <c r="D12" s="30"/>
+      <c r="E12" s="30"/>
     </row>
     <row r="13" spans="1:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
     <row r="14" spans="1:10" x14ac:dyDescent="0.25">
@@ -1021,17 +1024,17 @@
       <c r="J14" s="7"/>
     </row>
     <row r="15" spans="1:10" ht="21" x14ac:dyDescent="0.35">
-      <c r="B15" s="38" t="s">
+      <c r="B15" s="27" t="s">
         <v>9</v>
       </c>
-      <c r="C15" s="39"/>
-      <c r="D15" s="39"/>
-      <c r="E15" s="39"/>
-      <c r="F15" s="39"/>
-      <c r="G15" s="39"/>
-      <c r="H15" s="39"/>
-      <c r="I15" s="39"/>
-      <c r="J15" s="40"/>
+      <c r="C15" s="28"/>
+      <c r="D15" s="28"/>
+      <c r="E15" s="28"/>
+      <c r="F15" s="28"/>
+      <c r="G15" s="28"/>
+      <c r="H15" s="28"/>
+      <c r="I15" s="28"/>
+      <c r="J15" s="29"/>
     </row>
     <row r="16" spans="1:10" x14ac:dyDescent="0.25">
       <c r="B16" s="3"/>
@@ -1044,7 +1047,7 @@
       </c>
       <c r="D17" s="20"/>
       <c r="E17" s="10"/>
-      <c r="F17" s="12"/>
+      <c r="F17" s="43"/>
       <c r="G17" s="10"/>
       <c r="H17" s="10"/>
       <c r="I17" s="10"/>
@@ -1084,19 +1087,19 @@
         <v>19</v>
       </c>
       <c r="G20" s="23"/>
-      <c r="H20" s="33" t="s">
+      <c r="H20" s="38" t="s">
         <v>1</v>
       </c>
-      <c r="I20" s="33"/>
+      <c r="I20" s="38"/>
       <c r="J20" s="8"/>
     </row>
     <row r="21" spans="2:10" x14ac:dyDescent="0.25">
       <c r="B21" s="3"/>
-      <c r="C21" s="36" t="s">
+      <c r="C21" s="41" t="s">
         <v>2</v>
       </c>
-      <c r="D21" s="36"/>
-      <c r="E21" s="36"/>
+      <c r="D21" s="41"/>
+      <c r="E21" s="41"/>
       <c r="F21" s="24"/>
       <c r="G21" s="17"/>
       <c r="H21" s="25"/>
@@ -1105,11 +1108,11 @@
     </row>
     <row r="22" spans="2:10" x14ac:dyDescent="0.25">
       <c r="B22" s="3"/>
-      <c r="C22" s="35" t="s">
+      <c r="C22" s="40" t="s">
         <v>3</v>
       </c>
-      <c r="D22" s="35"/>
-      <c r="E22" s="35"/>
+      <c r="D22" s="40"/>
+      <c r="E22" s="40"/>
       <c r="F22" s="25"/>
       <c r="G22" s="16"/>
       <c r="H22" s="25"/>
@@ -1118,11 +1121,11 @@
     </row>
     <row r="23" spans="2:10" x14ac:dyDescent="0.25">
       <c r="B23" s="3"/>
-      <c r="C23" s="35" t="s">
+      <c r="C23" s="40" t="s">
         <v>4</v>
       </c>
-      <c r="D23" s="35"/>
-      <c r="E23" s="35"/>
+      <c r="D23" s="40"/>
+      <c r="E23" s="40"/>
       <c r="F23" s="25"/>
       <c r="G23" s="16"/>
       <c r="H23" s="25"/>
@@ -1131,11 +1134,11 @@
     </row>
     <row r="24" spans="2:10" x14ac:dyDescent="0.25">
       <c r="B24" s="3"/>
-      <c r="C24" s="29" t="s">
+      <c r="C24" s="34" t="s">
         <v>10</v>
       </c>
-      <c r="D24" s="29"/>
-      <c r="E24" s="29"/>
+      <c r="D24" s="34"/>
+      <c r="E24" s="34"/>
       <c r="F24" s="24"/>
       <c r="G24" s="17"/>
       <c r="H24" s="24"/>
@@ -1143,11 +1146,11 @@
     </row>
     <row r="25" spans="2:10" x14ac:dyDescent="0.25">
       <c r="B25" s="3"/>
-      <c r="C25" s="29" t="s">
+      <c r="C25" s="34" t="s">
         <v>11</v>
       </c>
-      <c r="D25" s="29"/>
-      <c r="E25" s="29"/>
+      <c r="D25" s="34"/>
+      <c r="E25" s="34"/>
       <c r="F25" s="24"/>
       <c r="G25" s="17"/>
       <c r="H25" s="24"/>
@@ -1155,11 +1158,11 @@
     </row>
     <row r="26" spans="2:10" x14ac:dyDescent="0.25">
       <c r="B26" s="3"/>
-      <c r="C26" s="37" t="s">
+      <c r="C26" s="42" t="s">
         <v>5</v>
       </c>
-      <c r="D26" s="37"/>
-      <c r="E26" s="37"/>
+      <c r="D26" s="42"/>
+      <c r="E26" s="42"/>
       <c r="F26" s="25"/>
       <c r="G26" s="16"/>
       <c r="H26" s="25"/>
@@ -1168,10 +1171,10 @@
     </row>
     <row r="27" spans="2:10" x14ac:dyDescent="0.25">
       <c r="B27" s="3"/>
-      <c r="C27" s="34" t="s">
+      <c r="C27" s="39" t="s">
         <v>12</v>
       </c>
-      <c r="D27" s="34"/>
+      <c r="D27" s="39"/>
       <c r="F27" s="24"/>
       <c r="G27" s="17"/>
       <c r="H27" s="24"/>
@@ -1190,10 +1193,10 @@
     </row>
     <row r="29" spans="2:10" x14ac:dyDescent="0.25">
       <c r="B29" s="3"/>
-      <c r="C29" s="35" t="s">
+      <c r="C29" s="40" t="s">
         <v>6</v>
       </c>
-      <c r="D29" s="35"/>
+      <c r="D29" s="40"/>
       <c r="E29" s="10"/>
       <c r="F29" s="25"/>
       <c r="G29" s="16"/>
@@ -1203,10 +1206,10 @@
     </row>
     <row r="30" spans="2:10" x14ac:dyDescent="0.25">
       <c r="B30" s="3"/>
-      <c r="C30" s="36" t="s">
+      <c r="C30" s="41" t="s">
         <v>7</v>
       </c>
-      <c r="D30" s="36"/>
+      <c r="D30" s="41"/>
       <c r="E30" s="10"/>
       <c r="F30" s="26"/>
       <c r="G30" s="18"/>
@@ -1226,61 +1229,56 @@
       <c r="J31" s="4"/>
     </row>
     <row r="32" spans="2:10" ht="31.9" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B32" s="30" t="s">
+      <c r="B32" s="35" t="s">
         <v>8</v>
       </c>
-      <c r="C32" s="31"/>
-      <c r="D32" s="31"/>
-      <c r="E32" s="31"/>
-      <c r="F32" s="31"/>
-      <c r="G32" s="31"/>
-      <c r="H32" s="31"/>
-      <c r="I32" s="31"/>
-      <c r="J32" s="32"/>
+      <c r="C32" s="36"/>
+      <c r="D32" s="36"/>
+      <c r="E32" s="36"/>
+      <c r="F32" s="36"/>
+      <c r="G32" s="36"/>
+      <c r="H32" s="36"/>
+      <c r="I32" s="36"/>
+      <c r="J32" s="37"/>
     </row>
     <row r="36" spans="2:10" ht="39.6" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="37" spans="2:10" x14ac:dyDescent="0.25">
-      <c r="B37" s="42"/>
-      <c r="C37" s="42"/>
-      <c r="D37" s="42"/>
-      <c r="E37" s="42"/>
-      <c r="F37" s="42"/>
-      <c r="G37" s="42"/>
-      <c r="H37" s="42"/>
-      <c r="I37" s="42"/>
-      <c r="J37" s="42"/>
+      <c r="B37" s="31"/>
+      <c r="C37" s="31"/>
+      <c r="D37" s="31"/>
+      <c r="E37" s="31"/>
+      <c r="F37" s="31"/>
+      <c r="G37" s="31"/>
+      <c r="H37" s="31"/>
+      <c r="I37" s="31"/>
+      <c r="J37" s="31"/>
     </row>
     <row r="38" spans="2:10" x14ac:dyDescent="0.25">
-      <c r="B38" s="27"/>
-      <c r="C38" s="27"/>
-      <c r="D38" s="27"/>
-      <c r="E38" s="27"/>
-      <c r="F38" s="27"/>
-      <c r="G38" s="27"/>
-      <c r="H38" s="27"/>
-      <c r="I38" s="27"/>
-      <c r="J38" s="27"/>
+      <c r="B38" s="32"/>
+      <c r="C38" s="32"/>
+      <c r="D38" s="32"/>
+      <c r="E38" s="32"/>
+      <c r="F38" s="32"/>
+      <c r="G38" s="32"/>
+      <c r="H38" s="32"/>
+      <c r="I38" s="32"/>
+      <c r="J38" s="32"/>
     </row>
     <row r="39" spans="2:10" x14ac:dyDescent="0.25">
-      <c r="B39" s="27"/>
-      <c r="C39" s="27"/>
-      <c r="D39" s="27"/>
-      <c r="E39" s="27"/>
-      <c r="F39" s="27"/>
-      <c r="G39" s="27"/>
-      <c r="H39" s="27"/>
-      <c r="I39" s="27"/>
-      <c r="J39" s="27"/>
+      <c r="B39" s="32"/>
+      <c r="C39" s="32"/>
+      <c r="D39" s="32"/>
+      <c r="E39" s="32"/>
+      <c r="F39" s="32"/>
+      <c r="G39" s="32"/>
+      <c r="H39" s="32"/>
+      <c r="I39" s="32"/>
+      <c r="J39" s="32"/>
     </row>
     <row r="44" spans="2:10" ht="58.15" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="46" spans="2:10" ht="59.45" customHeight="1" x14ac:dyDescent="0.25"/>
   </sheetData>
   <mergeCells count="19">
-    <mergeCell ref="B15:J15"/>
-    <mergeCell ref="B12:E12"/>
-    <mergeCell ref="B37:J37"/>
-    <mergeCell ref="B38:J38"/>
-    <mergeCell ref="B39:J39"/>
     <mergeCell ref="A4:J4"/>
     <mergeCell ref="A5:J5"/>
     <mergeCell ref="B10:J10"/>
@@ -1295,6 +1293,11 @@
     <mergeCell ref="C23:E23"/>
     <mergeCell ref="C22:E22"/>
     <mergeCell ref="C21:E21"/>
+    <mergeCell ref="B15:J15"/>
+    <mergeCell ref="B12:E12"/>
+    <mergeCell ref="B37:J37"/>
+    <mergeCell ref="B38:J38"/>
+    <mergeCell ref="B39:J39"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>

</xml_diff>

<commit_message>
Refactor NutrimentalExporter to adjust image sizes and positions; update cell writing logic for better layout
</commit_message>
<xml_diff>
--- a/templates/formato.xlsx
+++ b/templates/formato.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/e039d0c270e9facf/Desktop/Developer/UANL---LABORATORIO-DE-ALIMENTOS-MEDICAMENTOS-Y-TOXICOLOGIA/templates/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="110" documentId="8_{47FAC42F-AC07-43D6-8172-01CEADEBF0F6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{CF9D600E-358B-48D0-B18F-498332E19149}"/>
+  <xr:revisionPtr revIDLastSave="220" documentId="8_{47FAC42F-AC07-43D6-8172-01CEADEBF0F6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{D51EF4CC-1C71-4171-9674-747B8E5418E4}"/>
   <bookViews>
     <workbookView xWindow="-23148" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{1CB8A4CE-E91B-448F-9BE6-E546BA7C8907}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="20" uniqueCount="20">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="24" uniqueCount="23">
   <si>
     <t>1. TABLA DE INFORMACIÓN NUTRIMENTAL (DECLARACIÓN NUTRIMENTAL)</t>
   </si>
@@ -96,6 +96,27 @@
   </si>
   <si>
     <t>Por 100</t>
+  </si>
+  <si>
+    <t>2. SISTEMA DE ETIQUETADO FRONTAL</t>
+  </si>
+  <si>
+    <r>
+      <t>a) Información nutrimental complementaria.</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> Los sellos mostrados a continuación son los que aplican al producto analizado y deberán aparecer en ese orden en la etiqueta del producto. Si es más de un sello se deberá seguir la agrupación establecida por la norma NOM-051-SCFI/SSA1-2010.</t>
+    </r>
+  </si>
+  <si>
+    <t>Los productos cuya superficie principal de exhibición sea menor o igual a 40 cm² sólo deben incluir un sello con el número que corresponda a la cantidad de nutrimentos que cumplen con el perfil establecido en la tabla “A1-Tamaño de los sellos” del Apéndice A de la Norma NOM-051-SCFI/SSA1-2010 y deberá tener el tamaño establecido en el mismo documento el cual se puede descargar de internet usando las direcciones de página web mencionadas abajo. En aquellos productos cuya superficie principal de exhibición sea ≤ 5 cm² el octágono que indica el número de sellos (1 a 5 sellos) mencionado en el párrafo anterior deberá ajustarse a las dimensiones indicadas en el punto A4.4 del Apéndice A en la NOM-051-SCFI/SSA1-2010.</t>
   </si>
 </sst>
 </file>
@@ -350,7 +371,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="44">
+  <cellXfs count="47">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="right"/>
@@ -398,6 +419,42 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="13" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -416,38 +473,11 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right"/>
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="13" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -477,9 +507,9 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>10</xdr:col>
-      <xdr:colOff>624840</xdr:colOff>
+      <xdr:colOff>643890</xdr:colOff>
       <xdr:row>5</xdr:row>
-      <xdr:rowOff>94601</xdr:rowOff>
+      <xdr:rowOff>109841</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -540,7 +570,7 @@
       <xdr:col>11</xdr:col>
       <xdr:colOff>225597</xdr:colOff>
       <xdr:row>40</xdr:row>
-      <xdr:rowOff>167640</xdr:rowOff>
+      <xdr:rowOff>186690</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -572,6 +602,67 @@
         <a:xfrm>
           <a:off x="0" y="6686550"/>
           <a:ext cx="6580677" cy="1358265"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:noFill/>
+        <a:extLst>
+          <a:ext uri="{909E8E84-426E-40DD-AFC4-6F175D3DCCD1}">
+            <a14:hiddenFill xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main">
+              <a:solidFill>
+                <a:srgbClr val="FFFFFF"/>
+              </a:solidFill>
+            </a14:hiddenFill>
+          </a:ext>
+        </a:extLst>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>11</xdr:col>
+      <xdr:colOff>1</xdr:colOff>
+      <xdr:row>0</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>21</xdr:col>
+      <xdr:colOff>30480</xdr:colOff>
+      <xdr:row>5</xdr:row>
+      <xdr:rowOff>109843</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="2" name="Picture 1">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{C6E62307-5EB0-4CB0-9F1B-DC037290500A}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1" noChangeArrowheads="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill rotWithShape="1">
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId1">
+          <a:extLst>
+            <a:ext uri="{28A0092B-C50C-407E-A947-70E740481C1C}">
+              <a14:useLocalDpi xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" val="0"/>
+            </a:ext>
+          </a:extLst>
+        </a:blip>
+        <a:srcRect t="13298" b="19367"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr bwMode="auto">
+        <a:xfrm>
+          <a:off x="6454141" y="0"/>
+          <a:ext cx="5844539" cy="1062343"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -914,7 +1005,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{677BF1A9-BE92-4F6B-8063-3CDF98601680}">
-  <dimension ref="A4:J46"/>
+  <dimension ref="A4:U46"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="3" max="3" width="8.85546875" customWidth="1"/>
@@ -924,36 +1015,38 @@
     <col min="8" max="8" width="8.85546875" customWidth="1"/>
     <col min="9" max="9" width="3.42578125" customWidth="1"/>
     <col min="10" max="10" width="8.85546875" customWidth="1"/>
-    <col min="13" max="13" width="17.5703125" customWidth="1"/>
-    <col min="15" max="15" width="17.42578125" customWidth="1"/>
-    <col min="17" max="17" width="17.7109375" customWidth="1"/>
+    <col min="13" max="13" width="9.42578125" customWidth="1"/>
+    <col min="15" max="15" width="7.85546875" customWidth="1"/>
+    <col min="17" max="17" width="8.7109375" customWidth="1"/>
+    <col min="19" max="19" width="4.140625" customWidth="1"/>
+    <col min="20" max="20" width="5" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="4" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A4" s="33"/>
-      <c r="B4" s="33"/>
-      <c r="C4" s="33"/>
-      <c r="D4" s="33"/>
-      <c r="E4" s="33"/>
-      <c r="F4" s="33"/>
-      <c r="G4" s="33"/>
-      <c r="H4" s="33"/>
-      <c r="I4" s="33"/>
-      <c r="J4" s="33"/>
-    </row>
-    <row r="5" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A5" s="33"/>
-      <c r="B5" s="33"/>
-      <c r="C5" s="33"/>
-      <c r="D5" s="33"/>
-      <c r="E5" s="33"/>
-      <c r="F5" s="33"/>
-      <c r="G5" s="33"/>
-      <c r="H5" s="33"/>
-      <c r="I5" s="33"/>
-      <c r="J5" s="33"/>
-    </row>
-    <row r="6" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:21" x14ac:dyDescent="0.25">
+      <c r="A4" s="29"/>
+      <c r="B4" s="29"/>
+      <c r="C4" s="29"/>
+      <c r="D4" s="29"/>
+      <c r="E4" s="29"/>
+      <c r="F4" s="29"/>
+      <c r="G4" s="29"/>
+      <c r="H4" s="29"/>
+      <c r="I4" s="29"/>
+      <c r="J4" s="29"/>
+    </row>
+    <row r="5" spans="1:21" x14ac:dyDescent="0.25">
+      <c r="A5" s="29"/>
+      <c r="B5" s="29"/>
+      <c r="C5" s="29"/>
+      <c r="D5" s="29"/>
+      <c r="E5" s="29"/>
+      <c r="F5" s="29"/>
+      <c r="G5" s="29"/>
+      <c r="H5" s="29"/>
+      <c r="I5" s="29"/>
+      <c r="J5" s="29"/>
+    </row>
+    <row r="6" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A6" s="1"/>
       <c r="B6" s="1"/>
       <c r="C6" s="1"/>
@@ -965,7 +1058,7 @@
       <c r="I6" s="1"/>
       <c r="J6" s="1"/>
     </row>
-    <row r="7" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A7" s="1"/>
       <c r="B7" s="1"/>
       <c r="C7" s="1"/>
@@ -977,7 +1070,7 @@
       <c r="I7" s="1"/>
       <c r="J7" s="1"/>
     </row>
-    <row r="8" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:21" x14ac:dyDescent="0.25">
       <c r="B8" s="19" t="s">
         <v>18</v>
       </c>
@@ -989,30 +1082,68 @@
       <c r="H8" s="13"/>
       <c r="I8" s="13"/>
       <c r="J8" s="2"/>
-    </row>
-    <row r="10" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="B10" s="34" t="s">
+      <c r="M8" s="19" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="10" spans="1:21" x14ac:dyDescent="0.25">
+      <c r="B10" s="30" t="s">
         <v>0</v>
       </c>
-      <c r="C10" s="34"/>
-      <c r="D10" s="34"/>
-      <c r="E10" s="34"/>
-      <c r="F10" s="34"/>
-      <c r="G10" s="34"/>
-      <c r="H10" s="34"/>
-      <c r="I10" s="34"/>
-      <c r="J10" s="34"/>
-    </row>
-    <row r="12" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="B12" s="30" t="s">
+      <c r="C10" s="30"/>
+      <c r="D10" s="30"/>
+      <c r="E10" s="30"/>
+      <c r="F10" s="30"/>
+      <c r="G10" s="30"/>
+      <c r="H10" s="30"/>
+      <c r="I10" s="30"/>
+      <c r="J10" s="30"/>
+      <c r="M10" s="13" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="11" spans="1:21" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="M11" s="45" t="s">
+        <v>21</v>
+      </c>
+      <c r="N11" s="45"/>
+      <c r="O11" s="45"/>
+      <c r="P11" s="45"/>
+      <c r="Q11" s="45"/>
+      <c r="R11" s="45"/>
+      <c r="S11" s="45"/>
+      <c r="T11" s="45"/>
+      <c r="U11" s="45"/>
+    </row>
+    <row r="12" spans="1:21" x14ac:dyDescent="0.25">
+      <c r="B12" s="42" t="s">
         <v>17</v>
       </c>
-      <c r="C12" s="30"/>
-      <c r="D12" s="30"/>
-      <c r="E12" s="30"/>
-    </row>
-    <row r="13" spans="1:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
-    <row r="14" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="C12" s="42"/>
+      <c r="D12" s="42"/>
+      <c r="E12" s="42"/>
+      <c r="M12" s="45"/>
+      <c r="N12" s="45"/>
+      <c r="O12" s="45"/>
+      <c r="P12" s="45"/>
+      <c r="Q12" s="45"/>
+      <c r="R12" s="45"/>
+      <c r="S12" s="45"/>
+      <c r="T12" s="45"/>
+      <c r="U12" s="45"/>
+    </row>
+    <row r="13" spans="1:21" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="M13" s="45"/>
+      <c r="N13" s="45"/>
+      <c r="O13" s="45"/>
+      <c r="P13" s="45"/>
+      <c r="Q13" s="45"/>
+      <c r="R13" s="45"/>
+      <c r="S13" s="45"/>
+      <c r="T13" s="45"/>
+      <c r="U13" s="45"/>
+    </row>
+    <row r="14" spans="1:21" x14ac:dyDescent="0.25">
       <c r="B14" s="5"/>
       <c r="C14" s="6"/>
       <c r="D14" s="6"/>
@@ -1022,38 +1153,65 @@
       <c r="H14" s="6"/>
       <c r="I14" s="6"/>
       <c r="J14" s="7"/>
-    </row>
-    <row r="15" spans="1:10" ht="21" x14ac:dyDescent="0.35">
-      <c r="B15" s="27" t="s">
+      <c r="M14" s="45"/>
+      <c r="N14" s="45"/>
+      <c r="O14" s="45"/>
+      <c r="P14" s="45"/>
+      <c r="Q14" s="45"/>
+      <c r="R14" s="45"/>
+      <c r="S14" s="45"/>
+      <c r="T14" s="45"/>
+      <c r="U14" s="45"/>
+    </row>
+    <row r="15" spans="1:21" ht="21" x14ac:dyDescent="0.35">
+      <c r="B15" s="39" t="s">
         <v>9</v>
       </c>
-      <c r="C15" s="28"/>
-      <c r="D15" s="28"/>
-      <c r="E15" s="28"/>
-      <c r="F15" s="28"/>
-      <c r="G15" s="28"/>
-      <c r="H15" s="28"/>
-      <c r="I15" s="28"/>
-      <c r="J15" s="29"/>
-    </row>
-    <row r="16" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="C15" s="40"/>
+      <c r="D15" s="40"/>
+      <c r="E15" s="40"/>
+      <c r="F15" s="40"/>
+      <c r="G15" s="40"/>
+      <c r="H15" s="40"/>
+      <c r="I15" s="40"/>
+      <c r="J15" s="41"/>
+      <c r="M15" s="45"/>
+      <c r="N15" s="45"/>
+      <c r="O15" s="45"/>
+      <c r="P15" s="45"/>
+      <c r="Q15" s="45"/>
+      <c r="R15" s="45"/>
+      <c r="S15" s="45"/>
+      <c r="T15" s="45"/>
+      <c r="U15" s="45"/>
+    </row>
+    <row r="16" spans="1:21" x14ac:dyDescent="0.25">
       <c r="B16" s="3"/>
       <c r="J16" s="4"/>
-    </row>
-    <row r="17" spans="2:10" x14ac:dyDescent="0.25">
+      <c r="M16" s="45"/>
+      <c r="N16" s="45"/>
+      <c r="O16" s="45"/>
+      <c r="P16" s="45"/>
+      <c r="Q16" s="45"/>
+      <c r="R16" s="45"/>
+      <c r="S16" s="45"/>
+      <c r="T16" s="45"/>
+      <c r="U16" s="45"/>
+    </row>
+    <row r="17" spans="2:21" x14ac:dyDescent="0.25">
       <c r="B17" s="3"/>
       <c r="C17" s="20" t="s">
         <v>14</v>
       </c>
       <c r="D17" s="20"/>
       <c r="E17" s="10"/>
-      <c r="F17" s="43"/>
+      <c r="F17" s="27"/>
       <c r="G17" s="10"/>
       <c r="H17" s="10"/>
       <c r="I17" s="10"/>
       <c r="J17" s="4"/>
     </row>
-    <row r="18" spans="2:10" x14ac:dyDescent="0.25">
+    <row r="18" spans="2:21" x14ac:dyDescent="0.25">
       <c r="B18" s="3"/>
       <c r="C18" s="20" t="s">
         <v>15</v>
@@ -1065,7 +1223,7 @@
       <c r="I18" s="10"/>
       <c r="J18" s="4"/>
     </row>
-    <row r="19" spans="2:10" x14ac:dyDescent="0.25">
+    <row r="19" spans="2:21" x14ac:dyDescent="0.25">
       <c r="B19" s="3"/>
       <c r="C19" s="21" t="s">
         <v>16</v>
@@ -1078,7 +1236,7 @@
       <c r="I19" s="12"/>
       <c r="J19" s="4"/>
     </row>
-    <row r="20" spans="2:10" x14ac:dyDescent="0.25">
+    <row r="20" spans="2:21" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B20" s="3"/>
       <c r="C20" s="10"/>
       <c r="D20" s="10"/>
@@ -1087,100 +1245,165 @@
         <v>19</v>
       </c>
       <c r="G20" s="23"/>
-      <c r="H20" s="38" t="s">
+      <c r="H20" s="34" t="s">
         <v>1</v>
       </c>
-      <c r="I20" s="38"/>
+      <c r="I20" s="34"/>
       <c r="J20" s="8"/>
-    </row>
-    <row r="21" spans="2:10" x14ac:dyDescent="0.25">
+      <c r="N20" s="28"/>
+      <c r="O20" s="28"/>
+      <c r="P20" s="28"/>
+      <c r="Q20" s="28"/>
+      <c r="R20" s="28"/>
+    </row>
+    <row r="21" spans="2:21" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B21" s="3"/>
-      <c r="C21" s="41" t="s">
+      <c r="C21" s="37" t="s">
         <v>2</v>
       </c>
-      <c r="D21" s="41"/>
-      <c r="E21" s="41"/>
+      <c r="D21" s="37"/>
+      <c r="E21" s="37"/>
       <c r="F21" s="24"/>
       <c r="G21" s="17"/>
       <c r="H21" s="25"/>
       <c r="I21" s="10"/>
       <c r="J21" s="9"/>
-    </row>
-    <row r="22" spans="2:10" x14ac:dyDescent="0.25">
+      <c r="N21" s="28"/>
+      <c r="O21" s="28"/>
+      <c r="P21" s="28"/>
+      <c r="Q21" s="28"/>
+      <c r="R21" s="28"/>
+      <c r="S21" s="28"/>
+      <c r="T21" s="28"/>
+    </row>
+    <row r="22" spans="2:21" x14ac:dyDescent="0.25">
       <c r="B22" s="3"/>
-      <c r="C22" s="40" t="s">
+      <c r="C22" s="36" t="s">
         <v>3</v>
       </c>
-      <c r="D22" s="40"/>
-      <c r="E22" s="40"/>
+      <c r="D22" s="36"/>
+      <c r="E22" s="36"/>
       <c r="F22" s="25"/>
       <c r="G22" s="16"/>
       <c r="H22" s="25"/>
       <c r="I22" s="10"/>
       <c r="J22" s="8"/>
-    </row>
-    <row r="23" spans="2:10" x14ac:dyDescent="0.25">
+      <c r="M22" s="28"/>
+      <c r="N22" s="28"/>
+      <c r="O22" s="28"/>
+      <c r="P22" s="28"/>
+      <c r="Q22" s="28"/>
+      <c r="R22" s="28"/>
+      <c r="S22" s="28"/>
+      <c r="T22" s="28"/>
+    </row>
+    <row r="23" spans="2:21" x14ac:dyDescent="0.25">
       <c r="B23" s="3"/>
-      <c r="C23" s="40" t="s">
+      <c r="C23" s="36" t="s">
         <v>4</v>
       </c>
-      <c r="D23" s="40"/>
-      <c r="E23" s="40"/>
+      <c r="D23" s="36"/>
+      <c r="E23" s="36"/>
       <c r="F23" s="25"/>
       <c r="G23" s="16"/>
       <c r="H23" s="25"/>
       <c r="I23" s="10"/>
       <c r="J23" s="8"/>
-    </row>
-    <row r="24" spans="2:10" x14ac:dyDescent="0.25">
+      <c r="M23" s="28"/>
+      <c r="N23" s="28"/>
+      <c r="O23" s="28"/>
+      <c r="P23" s="28"/>
+      <c r="Q23" s="28"/>
+      <c r="R23" s="28"/>
+      <c r="S23" s="28"/>
+      <c r="T23" s="28"/>
+    </row>
+    <row r="24" spans="2:21" x14ac:dyDescent="0.25">
       <c r="B24" s="3"/>
-      <c r="C24" s="34" t="s">
+      <c r="C24" s="30" t="s">
         <v>10</v>
       </c>
-      <c r="D24" s="34"/>
-      <c r="E24" s="34"/>
+      <c r="D24" s="30"/>
+      <c r="E24" s="30"/>
       <c r="F24" s="24"/>
       <c r="G24" s="17"/>
       <c r="H24" s="24"/>
       <c r="J24" s="8"/>
-    </row>
-    <row r="25" spans="2:10" x14ac:dyDescent="0.25">
+      <c r="M24" s="28"/>
+      <c r="N24" s="28"/>
+      <c r="O24" s="28"/>
+      <c r="P24" s="28"/>
+      <c r="Q24" s="28"/>
+      <c r="R24" s="28"/>
+      <c r="S24" s="28"/>
+      <c r="T24" s="28"/>
+    </row>
+    <row r="25" spans="2:21" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B25" s="3"/>
-      <c r="C25" s="34" t="s">
+      <c r="C25" s="30" t="s">
         <v>11</v>
       </c>
-      <c r="D25" s="34"/>
-      <c r="E25" s="34"/>
+      <c r="D25" s="30"/>
+      <c r="E25" s="30"/>
       <c r="F25" s="24"/>
       <c r="G25" s="17"/>
       <c r="H25" s="24"/>
       <c r="J25" s="8"/>
-    </row>
-    <row r="26" spans="2:10" x14ac:dyDescent="0.25">
+      <c r="M25" s="46" t="s">
+        <v>22</v>
+      </c>
+      <c r="N25" s="46"/>
+      <c r="O25" s="46"/>
+      <c r="P25" s="46"/>
+      <c r="Q25" s="46"/>
+      <c r="R25" s="46"/>
+      <c r="S25" s="46"/>
+      <c r="T25" s="46"/>
+      <c r="U25" s="46"/>
+    </row>
+    <row r="26" spans="2:21" x14ac:dyDescent="0.25">
       <c r="B26" s="3"/>
-      <c r="C26" s="42" t="s">
+      <c r="C26" s="38" t="s">
         <v>5</v>
       </c>
-      <c r="D26" s="42"/>
-      <c r="E26" s="42"/>
+      <c r="D26" s="38"/>
+      <c r="E26" s="38"/>
       <c r="F26" s="25"/>
       <c r="G26" s="16"/>
       <c r="H26" s="25"/>
       <c r="I26" s="10"/>
       <c r="J26" s="8"/>
-    </row>
-    <row r="27" spans="2:10" x14ac:dyDescent="0.25">
+      <c r="M26" s="46"/>
+      <c r="N26" s="46"/>
+      <c r="O26" s="46"/>
+      <c r="P26" s="46"/>
+      <c r="Q26" s="46"/>
+      <c r="R26" s="46"/>
+      <c r="S26" s="46"/>
+      <c r="T26" s="46"/>
+      <c r="U26" s="46"/>
+    </row>
+    <row r="27" spans="2:21" x14ac:dyDescent="0.25">
       <c r="B27" s="3"/>
-      <c r="C27" s="39" t="s">
+      <c r="C27" s="35" t="s">
         <v>12</v>
       </c>
-      <c r="D27" s="39"/>
+      <c r="D27" s="35"/>
       <c r="F27" s="24"/>
       <c r="G27" s="17"/>
       <c r="H27" s="24"/>
       <c r="J27" s="8"/>
-    </row>
-    <row r="28" spans="2:10" x14ac:dyDescent="0.25">
+      <c r="M27" s="46"/>
+      <c r="N27" s="46"/>
+      <c r="O27" s="46"/>
+      <c r="P27" s="46"/>
+      <c r="Q27" s="46"/>
+      <c r="R27" s="46"/>
+      <c r="S27" s="46"/>
+      <c r="T27" s="46"/>
+      <c r="U27" s="46"/>
+    </row>
+    <row r="28" spans="2:21" x14ac:dyDescent="0.25">
       <c r="B28" s="3"/>
       <c r="C28" s="13" t="s">
         <v>13</v>
@@ -1190,34 +1413,61 @@
       <c r="G28" s="17"/>
       <c r="H28" s="24"/>
       <c r="J28" s="8"/>
-    </row>
-    <row r="29" spans="2:10" x14ac:dyDescent="0.25">
+      <c r="M28" s="46"/>
+      <c r="N28" s="46"/>
+      <c r="O28" s="46"/>
+      <c r="P28" s="46"/>
+      <c r="Q28" s="46"/>
+      <c r="R28" s="46"/>
+      <c r="S28" s="46"/>
+      <c r="T28" s="46"/>
+      <c r="U28" s="46"/>
+    </row>
+    <row r="29" spans="2:21" x14ac:dyDescent="0.25">
       <c r="B29" s="3"/>
-      <c r="C29" s="40" t="s">
+      <c r="C29" s="36" t="s">
         <v>6</v>
       </c>
-      <c r="D29" s="40"/>
+      <c r="D29" s="36"/>
       <c r="E29" s="10"/>
       <c r="F29" s="25"/>
       <c r="G29" s="16"/>
       <c r="H29" s="25"/>
       <c r="I29" s="10"/>
       <c r="J29" s="8"/>
-    </row>
-    <row r="30" spans="2:10" x14ac:dyDescent="0.25">
+      <c r="M29" s="46"/>
+      <c r="N29" s="46"/>
+      <c r="O29" s="46"/>
+      <c r="P29" s="46"/>
+      <c r="Q29" s="46"/>
+      <c r="R29" s="46"/>
+      <c r="S29" s="46"/>
+      <c r="T29" s="46"/>
+      <c r="U29" s="46"/>
+    </row>
+    <row r="30" spans="2:21" x14ac:dyDescent="0.25">
       <c r="B30" s="3"/>
-      <c r="C30" s="41" t="s">
+      <c r="C30" s="37" t="s">
         <v>7</v>
       </c>
-      <c r="D30" s="41"/>
+      <c r="D30" s="37"/>
       <c r="E30" s="10"/>
       <c r="F30" s="26"/>
       <c r="G30" s="18"/>
       <c r="H30" s="26"/>
       <c r="I30" s="12"/>
       <c r="J30" s="8"/>
-    </row>
-    <row r="31" spans="2:10" x14ac:dyDescent="0.25">
+      <c r="M30" s="46"/>
+      <c r="N30" s="46"/>
+      <c r="O30" s="46"/>
+      <c r="P30" s="46"/>
+      <c r="Q30" s="46"/>
+      <c r="R30" s="46"/>
+      <c r="S30" s="46"/>
+      <c r="T30" s="46"/>
+      <c r="U30" s="46"/>
+    </row>
+    <row r="31" spans="2:21" x14ac:dyDescent="0.25">
       <c r="B31" s="3"/>
       <c r="C31" s="10"/>
       <c r="D31" s="10"/>
@@ -1227,58 +1477,124 @@
       <c r="H31" s="10"/>
       <c r="I31" s="10"/>
       <c r="J31" s="4"/>
-    </row>
-    <row r="32" spans="2:10" ht="31.9" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B32" s="35" t="s">
+      <c r="M31" s="46"/>
+      <c r="N31" s="46"/>
+      <c r="O31" s="46"/>
+      <c r="P31" s="46"/>
+      <c r="Q31" s="46"/>
+      <c r="R31" s="46"/>
+      <c r="S31" s="46"/>
+      <c r="T31" s="46"/>
+      <c r="U31" s="46"/>
+    </row>
+    <row r="32" spans="2:21" ht="31.9" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B32" s="31" t="s">
         <v>8</v>
       </c>
-      <c r="C32" s="36"/>
-      <c r="D32" s="36"/>
-      <c r="E32" s="36"/>
-      <c r="F32" s="36"/>
-      <c r="G32" s="36"/>
-      <c r="H32" s="36"/>
-      <c r="I32" s="36"/>
-      <c r="J32" s="37"/>
-    </row>
-    <row r="36" spans="2:10" ht="39.6" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="37" spans="2:10" x14ac:dyDescent="0.25">
-      <c r="B37" s="31"/>
-      <c r="C37" s="31"/>
-      <c r="D37" s="31"/>
-      <c r="E37" s="31"/>
-      <c r="F37" s="31"/>
-      <c r="G37" s="31"/>
-      <c r="H37" s="31"/>
-      <c r="I37" s="31"/>
-      <c r="J37" s="31"/>
-    </row>
-    <row r="38" spans="2:10" x14ac:dyDescent="0.25">
-      <c r="B38" s="32"/>
-      <c r="C38" s="32"/>
-      <c r="D38" s="32"/>
-      <c r="E38" s="32"/>
-      <c r="F38" s="32"/>
-      <c r="G38" s="32"/>
-      <c r="H38" s="32"/>
-      <c r="I38" s="32"/>
-      <c r="J38" s="32"/>
-    </row>
-    <row r="39" spans="2:10" x14ac:dyDescent="0.25">
-      <c r="B39" s="32"/>
-      <c r="C39" s="32"/>
-      <c r="D39" s="32"/>
-      <c r="E39" s="32"/>
-      <c r="F39" s="32"/>
-      <c r="G39" s="32"/>
-      <c r="H39" s="32"/>
-      <c r="I39" s="32"/>
-      <c r="J39" s="32"/>
-    </row>
-    <row r="44" spans="2:10" ht="58.15" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="46" spans="2:10" ht="59.45" customHeight="1" x14ac:dyDescent="0.25"/>
+      <c r="C32" s="32"/>
+      <c r="D32" s="32"/>
+      <c r="E32" s="32"/>
+      <c r="F32" s="32"/>
+      <c r="G32" s="32"/>
+      <c r="H32" s="32"/>
+      <c r="I32" s="32"/>
+      <c r="J32" s="33"/>
+      <c r="M32" s="46"/>
+      <c r="N32" s="46"/>
+      <c r="O32" s="46"/>
+      <c r="P32" s="46"/>
+      <c r="Q32" s="46"/>
+      <c r="R32" s="46"/>
+      <c r="S32" s="46"/>
+      <c r="T32" s="46"/>
+      <c r="U32" s="46"/>
+    </row>
+    <row r="33" spans="2:21" x14ac:dyDescent="0.25">
+      <c r="M33" s="46"/>
+      <c r="N33" s="46"/>
+      <c r="O33" s="46"/>
+      <c r="P33" s="46"/>
+      <c r="Q33" s="46"/>
+      <c r="R33" s="46"/>
+      <c r="S33" s="46"/>
+      <c r="T33" s="46"/>
+      <c r="U33" s="46"/>
+    </row>
+    <row r="34" spans="2:21" x14ac:dyDescent="0.25">
+      <c r="M34" s="46"/>
+      <c r="N34" s="46"/>
+      <c r="O34" s="46"/>
+      <c r="P34" s="46"/>
+      <c r="Q34" s="46"/>
+      <c r="R34" s="46"/>
+      <c r="S34" s="46"/>
+      <c r="T34" s="46"/>
+      <c r="U34" s="46"/>
+    </row>
+    <row r="35" spans="2:21" x14ac:dyDescent="0.25">
+      <c r="M35" s="46"/>
+      <c r="N35" s="46"/>
+      <c r="O35" s="46"/>
+      <c r="P35" s="46"/>
+      <c r="Q35" s="46"/>
+      <c r="R35" s="46"/>
+      <c r="S35" s="46"/>
+      <c r="T35" s="46"/>
+      <c r="U35" s="46"/>
+    </row>
+    <row r="36" spans="2:21" ht="39.6" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="M36" s="46"/>
+      <c r="N36" s="46"/>
+      <c r="O36" s="46"/>
+      <c r="P36" s="46"/>
+      <c r="Q36" s="46"/>
+      <c r="R36" s="46"/>
+      <c r="S36" s="46"/>
+      <c r="T36" s="46"/>
+      <c r="U36" s="46"/>
+    </row>
+    <row r="37" spans="2:21" x14ac:dyDescent="0.25">
+      <c r="B37" s="43"/>
+      <c r="C37" s="43"/>
+      <c r="D37" s="43"/>
+      <c r="E37" s="43"/>
+      <c r="F37" s="43"/>
+      <c r="G37" s="43"/>
+      <c r="H37" s="43"/>
+      <c r="I37" s="43"/>
+      <c r="J37" s="43"/>
+    </row>
+    <row r="38" spans="2:21" x14ac:dyDescent="0.25">
+      <c r="B38" s="44"/>
+      <c r="C38" s="44"/>
+      <c r="D38" s="44"/>
+      <c r="E38" s="44"/>
+      <c r="F38" s="44"/>
+      <c r="G38" s="44"/>
+      <c r="H38" s="44"/>
+      <c r="I38" s="44"/>
+      <c r="J38" s="44"/>
+    </row>
+    <row r="39" spans="2:21" x14ac:dyDescent="0.25">
+      <c r="B39" s="44"/>
+      <c r="C39" s="44"/>
+      <c r="D39" s="44"/>
+      <c r="E39" s="44"/>
+      <c r="F39" s="44"/>
+      <c r="G39" s="44"/>
+      <c r="H39" s="44"/>
+      <c r="I39" s="44"/>
+      <c r="J39" s="44"/>
+    </row>
+    <row r="44" spans="2:21" ht="58.15" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="46" spans="2:21" ht="59.45" customHeight="1" x14ac:dyDescent="0.25"/>
   </sheetData>
-  <mergeCells count="19">
+  <mergeCells count="21">
+    <mergeCell ref="B37:J37"/>
+    <mergeCell ref="B38:J38"/>
+    <mergeCell ref="B39:J39"/>
+    <mergeCell ref="M11:U16"/>
+    <mergeCell ref="M25:U36"/>
     <mergeCell ref="A4:J4"/>
     <mergeCell ref="A5:J5"/>
     <mergeCell ref="B10:J10"/>
@@ -1295,9 +1611,6 @@
     <mergeCell ref="C21:E21"/>
     <mergeCell ref="B15:J15"/>
     <mergeCell ref="B12:E12"/>
-    <mergeCell ref="B37:J37"/>
-    <mergeCell ref="B38:J38"/>
-    <mergeCell ref="B39:J39"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>

</xml_diff>

<commit_message>
Refactor NutrimentalModule to combine energy content display; enhance column sizing and formatting for nutritional table
</commit_message>
<xml_diff>
--- a/templates/formato.xlsx
+++ b/templates/formato.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29231"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29328"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/e039d0c270e9facf/Desktop/Developer/UANL---LABORATORIO-DE-ALIMENTOS-MEDICAMENTOS-Y-TOXICOLOGIA/templates/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="220" documentId="8_{47FAC42F-AC07-43D6-8172-01CEADEBF0F6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{D51EF4CC-1C71-4171-9674-747B8E5418E4}"/>
+  <xr:revisionPtr revIDLastSave="283" documentId="8_{47FAC42F-AC07-43D6-8172-01CEADEBF0F6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{AB47CCD7-2A7F-430E-B7B5-7AC47D685782}"/>
   <bookViews>
-    <workbookView xWindow="-23148" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{1CB8A4CE-E91B-448F-9BE6-E546BA7C8907}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{1CB8A4CE-E91B-448F-9BE6-E546BA7C8907}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -507,9 +507,9 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>10</xdr:col>
-      <xdr:colOff>643890</xdr:colOff>
+      <xdr:colOff>19050</xdr:colOff>
       <xdr:row>5</xdr:row>
-      <xdr:rowOff>109841</xdr:rowOff>
+      <xdr:rowOff>58947</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -540,7 +540,7 @@
       <xdr:spPr bwMode="auto">
         <a:xfrm>
           <a:off x="0" y="7618"/>
-          <a:ext cx="6362700" cy="1001383"/>
+          <a:ext cx="6124575" cy="1003829"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -568,7 +568,7 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>11</xdr:col>
-      <xdr:colOff>225597</xdr:colOff>
+      <xdr:colOff>216072</xdr:colOff>
       <xdr:row>40</xdr:row>
       <xdr:rowOff>186690</xdr:rowOff>
     </xdr:to>
@@ -622,16 +622,16 @@
   </xdr:twoCellAnchor>
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
-      <xdr:col>11</xdr:col>
-      <xdr:colOff>1</xdr:colOff>
+      <xdr:col>10</xdr:col>
+      <xdr:colOff>200027</xdr:colOff>
       <xdr:row>0</xdr:row>
-      <xdr:rowOff>0</xdr:rowOff>
+      <xdr:rowOff>1</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>21</xdr:col>
-      <xdr:colOff>30480</xdr:colOff>
+      <xdr:col>20</xdr:col>
+      <xdr:colOff>140865</xdr:colOff>
       <xdr:row>5</xdr:row>
-      <xdr:rowOff>109843</xdr:rowOff>
+      <xdr:rowOff>38101</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -661,8 +661,8 @@
       </xdr:blipFill>
       <xdr:spPr bwMode="auto">
         <a:xfrm>
-          <a:off x="6454141" y="0"/>
-          <a:ext cx="5844539" cy="1062343"/>
+          <a:off x="6315077" y="1"/>
+          <a:ext cx="5446288" cy="990600"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -1005,24 +1005,27 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{677BF1A9-BE92-4F6B-8063-3CDF98601680}">
-  <dimension ref="A4:U46"/>
+  <dimension ref="A4:T46"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
+    <col min="2" max="2" width="3.7109375" customWidth="1"/>
     <col min="3" max="3" width="8.85546875" customWidth="1"/>
     <col min="4" max="4" width="9.28515625" customWidth="1"/>
-    <col min="6" max="6" width="8.85546875" customWidth="1"/>
-    <col min="7" max="7" width="4.85546875" customWidth="1"/>
-    <col min="8" max="8" width="8.85546875" customWidth="1"/>
-    <col min="9" max="9" width="3.42578125" customWidth="1"/>
-    <col min="10" max="10" width="8.85546875" customWidth="1"/>
-    <col min="13" max="13" width="9.42578125" customWidth="1"/>
-    <col min="15" max="15" width="7.85546875" customWidth="1"/>
-    <col min="17" max="17" width="8.7109375" customWidth="1"/>
-    <col min="19" max="19" width="4.140625" customWidth="1"/>
-    <col min="20" max="20" width="5" customWidth="1"/>
+    <col min="5" max="5" width="6.85546875" customWidth="1"/>
+    <col min="6" max="6" width="17.5703125" customWidth="1"/>
+    <col min="7" max="7" width="3.42578125" customWidth="1"/>
+    <col min="8" max="8" width="18.7109375" customWidth="1"/>
+    <col min="9" max="9" width="3.5703125" customWidth="1"/>
+    <col min="10" max="10" width="3.85546875" customWidth="1"/>
+    <col min="11" max="11" width="4.85546875" customWidth="1"/>
+    <col min="12" max="12" width="9.42578125" customWidth="1"/>
+    <col min="14" max="14" width="7.85546875" customWidth="1"/>
+    <col min="16" max="16" width="8.7109375" customWidth="1"/>
+    <col min="18" max="18" width="4.140625" customWidth="1"/>
+    <col min="19" max="19" width="5" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="4" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A4" s="29"/>
       <c r="B4" s="29"/>
       <c r="C4" s="29"/>
@@ -1034,7 +1037,7 @@
       <c r="I4" s="29"/>
       <c r="J4" s="29"/>
     </row>
-    <row r="5" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A5" s="29"/>
       <c r="B5" s="29"/>
       <c r="C5" s="29"/>
@@ -1046,7 +1049,7 @@
       <c r="I5" s="29"/>
       <c r="J5" s="29"/>
     </row>
-    <row r="6" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A6" s="1"/>
       <c r="B6" s="1"/>
       <c r="C6" s="1"/>
@@ -1058,7 +1061,7 @@
       <c r="I6" s="1"/>
       <c r="J6" s="1"/>
     </row>
-    <row r="7" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A7" s="1"/>
       <c r="B7" s="1"/>
       <c r="C7" s="1"/>
@@ -1070,7 +1073,7 @@
       <c r="I7" s="1"/>
       <c r="J7" s="1"/>
     </row>
-    <row r="8" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:20" x14ac:dyDescent="0.25">
       <c r="B8" s="19" t="s">
         <v>18</v>
       </c>
@@ -1082,11 +1085,11 @@
       <c r="H8" s="13"/>
       <c r="I8" s="13"/>
       <c r="J8" s="2"/>
-      <c r="M8" s="19" t="s">
+      <c r="L8" s="19" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="10" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:20" x14ac:dyDescent="0.25">
       <c r="B10" s="30" t="s">
         <v>0</v>
       </c>
@@ -1098,14 +1101,15 @@
       <c r="H10" s="30"/>
       <c r="I10" s="30"/>
       <c r="J10" s="30"/>
-      <c r="M10" s="13" t="s">
+      <c r="L10" s="13" t="s">
         <v>20</v>
       </c>
     </row>
-    <row r="11" spans="1:21" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="M11" s="45" t="s">
+    <row r="11" spans="1:20" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="L11" s="45" t="s">
         <v>21</v>
       </c>
+      <c r="M11" s="45"/>
       <c r="N11" s="45"/>
       <c r="O11" s="45"/>
       <c r="P11" s="45"/>
@@ -1113,15 +1117,15 @@
       <c r="R11" s="45"/>
       <c r="S11" s="45"/>
       <c r="T11" s="45"/>
-      <c r="U11" s="45"/>
-    </row>
-    <row r="12" spans="1:21" x14ac:dyDescent="0.25">
+    </row>
+    <row r="12" spans="1:20" x14ac:dyDescent="0.25">
       <c r="B12" s="42" t="s">
         <v>17</v>
       </c>
       <c r="C12" s="42"/>
       <c r="D12" s="42"/>
       <c r="E12" s="42"/>
+      <c r="L12" s="45"/>
       <c r="M12" s="45"/>
       <c r="N12" s="45"/>
       <c r="O12" s="45"/>
@@ -1130,9 +1134,9 @@
       <c r="R12" s="45"/>
       <c r="S12" s="45"/>
       <c r="T12" s="45"/>
-      <c r="U12" s="45"/>
-    </row>
-    <row r="13" spans="1:21" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    </row>
+    <row r="13" spans="1:20" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="L13" s="45"/>
       <c r="M13" s="45"/>
       <c r="N13" s="45"/>
       <c r="O13" s="45"/>
@@ -1141,9 +1145,8 @@
       <c r="R13" s="45"/>
       <c r="S13" s="45"/>
       <c r="T13" s="45"/>
-      <c r="U13" s="45"/>
-    </row>
-    <row r="14" spans="1:21" x14ac:dyDescent="0.25">
+    </row>
+    <row r="14" spans="1:20" x14ac:dyDescent="0.25">
       <c r="B14" s="5"/>
       <c r="C14" s="6"/>
       <c r="D14" s="6"/>
@@ -1153,6 +1156,7 @@
       <c r="H14" s="6"/>
       <c r="I14" s="6"/>
       <c r="J14" s="7"/>
+      <c r="L14" s="45"/>
       <c r="M14" s="45"/>
       <c r="N14" s="45"/>
       <c r="O14" s="45"/>
@@ -1161,9 +1165,8 @@
       <c r="R14" s="45"/>
       <c r="S14" s="45"/>
       <c r="T14" s="45"/>
-      <c r="U14" s="45"/>
-    </row>
-    <row r="15" spans="1:21" ht="21" x14ac:dyDescent="0.35">
+    </row>
+    <row r="15" spans="1:20" ht="21" x14ac:dyDescent="0.35">
       <c r="B15" s="39" t="s">
         <v>9</v>
       </c>
@@ -1175,6 +1178,7 @@
       <c r="H15" s="40"/>
       <c r="I15" s="40"/>
       <c r="J15" s="41"/>
+      <c r="L15" s="45"/>
       <c r="M15" s="45"/>
       <c r="N15" s="45"/>
       <c r="O15" s="45"/>
@@ -1183,11 +1187,11 @@
       <c r="R15" s="45"/>
       <c r="S15" s="45"/>
       <c r="T15" s="45"/>
-      <c r="U15" s="45"/>
-    </row>
-    <row r="16" spans="1:21" x14ac:dyDescent="0.25">
+    </row>
+    <row r="16" spans="1:20" x14ac:dyDescent="0.25">
       <c r="B16" s="3"/>
       <c r="J16" s="4"/>
+      <c r="L16" s="45"/>
       <c r="M16" s="45"/>
       <c r="N16" s="45"/>
       <c r="O16" s="45"/>
@@ -1196,9 +1200,8 @@
       <c r="R16" s="45"/>
       <c r="S16" s="45"/>
       <c r="T16" s="45"/>
-      <c r="U16" s="45"/>
-    </row>
-    <row r="17" spans="2:21" x14ac:dyDescent="0.25">
+    </row>
+    <row r="17" spans="2:20" x14ac:dyDescent="0.25">
       <c r="B17" s="3"/>
       <c r="C17" s="20" t="s">
         <v>14</v>
@@ -1211,7 +1214,7 @@
       <c r="I17" s="10"/>
       <c r="J17" s="4"/>
     </row>
-    <row r="18" spans="2:21" x14ac:dyDescent="0.25">
+    <row r="18" spans="2:20" x14ac:dyDescent="0.25">
       <c r="B18" s="3"/>
       <c r="C18" s="20" t="s">
         <v>15</v>
@@ -1223,7 +1226,7 @@
       <c r="I18" s="10"/>
       <c r="J18" s="4"/>
     </row>
-    <row r="19" spans="2:21" x14ac:dyDescent="0.25">
+    <row r="19" spans="2:20" x14ac:dyDescent="0.25">
       <c r="B19" s="3"/>
       <c r="C19" s="21" t="s">
         <v>16</v>
@@ -1236,7 +1239,7 @@
       <c r="I19" s="12"/>
       <c r="J19" s="4"/>
     </row>
-    <row r="20" spans="2:21" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="20" spans="2:20" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B20" s="3"/>
       <c r="C20" s="10"/>
       <c r="D20" s="10"/>
@@ -1250,13 +1253,13 @@
       </c>
       <c r="I20" s="34"/>
       <c r="J20" s="8"/>
+      <c r="M20" s="28"/>
       <c r="N20" s="28"/>
       <c r="O20" s="28"/>
       <c r="P20" s="28"/>
       <c r="Q20" s="28"/>
-      <c r="R20" s="28"/>
-    </row>
-    <row r="21" spans="2:21" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    </row>
+    <row r="21" spans="2:20" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B21" s="3"/>
       <c r="C21" s="37" t="s">
         <v>2</v>
@@ -1268,15 +1271,15 @@
       <c r="H21" s="25"/>
       <c r="I21" s="10"/>
       <c r="J21" s="9"/>
+      <c r="M21" s="28"/>
       <c r="N21" s="28"/>
       <c r="O21" s="28"/>
       <c r="P21" s="28"/>
       <c r="Q21" s="28"/>
       <c r="R21" s="28"/>
       <c r="S21" s="28"/>
-      <c r="T21" s="28"/>
-    </row>
-    <row r="22" spans="2:21" x14ac:dyDescent="0.25">
+    </row>
+    <row r="22" spans="2:20" x14ac:dyDescent="0.25">
       <c r="B22" s="3"/>
       <c r="C22" s="36" t="s">
         <v>3</v>
@@ -1288,6 +1291,7 @@
       <c r="H22" s="25"/>
       <c r="I22" s="10"/>
       <c r="J22" s="8"/>
+      <c r="L22" s="28"/>
       <c r="M22" s="28"/>
       <c r="N22" s="28"/>
       <c r="O22" s="28"/>
@@ -1295,9 +1299,8 @@
       <c r="Q22" s="28"/>
       <c r="R22" s="28"/>
       <c r="S22" s="28"/>
-      <c r="T22" s="28"/>
-    </row>
-    <row r="23" spans="2:21" x14ac:dyDescent="0.25">
+    </row>
+    <row r="23" spans="2:20" x14ac:dyDescent="0.25">
       <c r="B23" s="3"/>
       <c r="C23" s="36" t="s">
         <v>4</v>
@@ -1309,6 +1312,7 @@
       <c r="H23" s="25"/>
       <c r="I23" s="10"/>
       <c r="J23" s="8"/>
+      <c r="L23" s="28"/>
       <c r="M23" s="28"/>
       <c r="N23" s="28"/>
       <c r="O23" s="28"/>
@@ -1316,9 +1320,8 @@
       <c r="Q23" s="28"/>
       <c r="R23" s="28"/>
       <c r="S23" s="28"/>
-      <c r="T23" s="28"/>
-    </row>
-    <row r="24" spans="2:21" x14ac:dyDescent="0.25">
+    </row>
+    <row r="24" spans="2:20" x14ac:dyDescent="0.25">
       <c r="B24" s="3"/>
       <c r="C24" s="30" t="s">
         <v>10</v>
@@ -1329,6 +1332,7 @@
       <c r="G24" s="17"/>
       <c r="H24" s="24"/>
       <c r="J24" s="8"/>
+      <c r="L24" s="28"/>
       <c r="M24" s="28"/>
       <c r="N24" s="28"/>
       <c r="O24" s="28"/>
@@ -1336,9 +1340,8 @@
       <c r="Q24" s="28"/>
       <c r="R24" s="28"/>
       <c r="S24" s="28"/>
-      <c r="T24" s="28"/>
-    </row>
-    <row r="25" spans="2:21" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    </row>
+    <row r="25" spans="2:20" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B25" s="3"/>
       <c r="C25" s="30" t="s">
         <v>11</v>
@@ -1349,9 +1352,10 @@
       <c r="G25" s="17"/>
       <c r="H25" s="24"/>
       <c r="J25" s="8"/>
-      <c r="M25" s="46" t="s">
+      <c r="L25" s="46" t="s">
         <v>22</v>
       </c>
+      <c r="M25" s="46"/>
       <c r="N25" s="46"/>
       <c r="O25" s="46"/>
       <c r="P25" s="46"/>
@@ -1359,9 +1363,8 @@
       <c r="R25" s="46"/>
       <c r="S25" s="46"/>
       <c r="T25" s="46"/>
-      <c r="U25" s="46"/>
-    </row>
-    <row r="26" spans="2:21" x14ac:dyDescent="0.25">
+    </row>
+    <row r="26" spans="2:20" x14ac:dyDescent="0.25">
       <c r="B26" s="3"/>
       <c r="C26" s="38" t="s">
         <v>5</v>
@@ -1373,6 +1376,7 @@
       <c r="H26" s="25"/>
       <c r="I26" s="10"/>
       <c r="J26" s="8"/>
+      <c r="L26" s="46"/>
       <c r="M26" s="46"/>
       <c r="N26" s="46"/>
       <c r="O26" s="46"/>
@@ -1381,9 +1385,8 @@
       <c r="R26" s="46"/>
       <c r="S26" s="46"/>
       <c r="T26" s="46"/>
-      <c r="U26" s="46"/>
-    </row>
-    <row r="27" spans="2:21" x14ac:dyDescent="0.25">
+    </row>
+    <row r="27" spans="2:20" x14ac:dyDescent="0.25">
       <c r="B27" s="3"/>
       <c r="C27" s="35" t="s">
         <v>12</v>
@@ -1393,6 +1396,7 @@
       <c r="G27" s="17"/>
       <c r="H27" s="24"/>
       <c r="J27" s="8"/>
+      <c r="L27" s="46"/>
       <c r="M27" s="46"/>
       <c r="N27" s="46"/>
       <c r="O27" s="46"/>
@@ -1401,9 +1405,8 @@
       <c r="R27" s="46"/>
       <c r="S27" s="46"/>
       <c r="T27" s="46"/>
-      <c r="U27" s="46"/>
-    </row>
-    <row r="28" spans="2:21" x14ac:dyDescent="0.25">
+    </row>
+    <row r="28" spans="2:20" x14ac:dyDescent="0.25">
       <c r="B28" s="3"/>
       <c r="C28" s="13" t="s">
         <v>13</v>
@@ -1413,6 +1416,7 @@
       <c r="G28" s="17"/>
       <c r="H28" s="24"/>
       <c r="J28" s="8"/>
+      <c r="L28" s="46"/>
       <c r="M28" s="46"/>
       <c r="N28" s="46"/>
       <c r="O28" s="46"/>
@@ -1421,9 +1425,8 @@
       <c r="R28" s="46"/>
       <c r="S28" s="46"/>
       <c r="T28" s="46"/>
-      <c r="U28" s="46"/>
-    </row>
-    <row r="29" spans="2:21" x14ac:dyDescent="0.25">
+    </row>
+    <row r="29" spans="2:20" x14ac:dyDescent="0.25">
       <c r="B29" s="3"/>
       <c r="C29" s="36" t="s">
         <v>6</v>
@@ -1435,6 +1438,7 @@
       <c r="H29" s="25"/>
       <c r="I29" s="10"/>
       <c r="J29" s="8"/>
+      <c r="L29" s="46"/>
       <c r="M29" s="46"/>
       <c r="N29" s="46"/>
       <c r="O29" s="46"/>
@@ -1443,9 +1447,8 @@
       <c r="R29" s="46"/>
       <c r="S29" s="46"/>
       <c r="T29" s="46"/>
-      <c r="U29" s="46"/>
-    </row>
-    <row r="30" spans="2:21" x14ac:dyDescent="0.25">
+    </row>
+    <row r="30" spans="2:20" x14ac:dyDescent="0.25">
       <c r="B30" s="3"/>
       <c r="C30" s="37" t="s">
         <v>7</v>
@@ -1457,6 +1460,7 @@
       <c r="H30" s="26"/>
       <c r="I30" s="12"/>
       <c r="J30" s="8"/>
+      <c r="L30" s="46"/>
       <c r="M30" s="46"/>
       <c r="N30" s="46"/>
       <c r="O30" s="46"/>
@@ -1465,9 +1469,8 @@
       <c r="R30" s="46"/>
       <c r="S30" s="46"/>
       <c r="T30" s="46"/>
-      <c r="U30" s="46"/>
-    </row>
-    <row r="31" spans="2:21" x14ac:dyDescent="0.25">
+    </row>
+    <row r="31" spans="2:20" x14ac:dyDescent="0.25">
       <c r="B31" s="3"/>
       <c r="C31" s="10"/>
       <c r="D31" s="10"/>
@@ -1477,6 +1480,7 @@
       <c r="H31" s="10"/>
       <c r="I31" s="10"/>
       <c r="J31" s="4"/>
+      <c r="L31" s="46"/>
       <c r="M31" s="46"/>
       <c r="N31" s="46"/>
       <c r="O31" s="46"/>
@@ -1485,9 +1489,8 @@
       <c r="R31" s="46"/>
       <c r="S31" s="46"/>
       <c r="T31" s="46"/>
-      <c r="U31" s="46"/>
-    </row>
-    <row r="32" spans="2:21" ht="31.9" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    </row>
+    <row r="32" spans="2:20" ht="31.9" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B32" s="31" t="s">
         <v>8</v>
       </c>
@@ -1499,6 +1502,7 @@
       <c r="H32" s="32"/>
       <c r="I32" s="32"/>
       <c r="J32" s="33"/>
+      <c r="L32" s="46"/>
       <c r="M32" s="46"/>
       <c r="N32" s="46"/>
       <c r="O32" s="46"/>
@@ -1507,9 +1511,9 @@
       <c r="R32" s="46"/>
       <c r="S32" s="46"/>
       <c r="T32" s="46"/>
-      <c r="U32" s="46"/>
-    </row>
-    <row r="33" spans="2:21" x14ac:dyDescent="0.25">
+    </row>
+    <row r="33" spans="2:20" x14ac:dyDescent="0.25">
+      <c r="L33" s="46"/>
       <c r="M33" s="46"/>
       <c r="N33" s="46"/>
       <c r="O33" s="46"/>
@@ -1518,9 +1522,9 @@
       <c r="R33" s="46"/>
       <c r="S33" s="46"/>
       <c r="T33" s="46"/>
-      <c r="U33" s="46"/>
-    </row>
-    <row r="34" spans="2:21" x14ac:dyDescent="0.25">
+    </row>
+    <row r="34" spans="2:20" x14ac:dyDescent="0.25">
+      <c r="L34" s="46"/>
       <c r="M34" s="46"/>
       <c r="N34" s="46"/>
       <c r="O34" s="46"/>
@@ -1529,9 +1533,9 @@
       <c r="R34" s="46"/>
       <c r="S34" s="46"/>
       <c r="T34" s="46"/>
-      <c r="U34" s="46"/>
-    </row>
-    <row r="35" spans="2:21" x14ac:dyDescent="0.25">
+    </row>
+    <row r="35" spans="2:20" x14ac:dyDescent="0.25">
+      <c r="L35" s="46"/>
       <c r="M35" s="46"/>
       <c r="N35" s="46"/>
       <c r="O35" s="46"/>
@@ -1540,9 +1544,9 @@
       <c r="R35" s="46"/>
       <c r="S35" s="46"/>
       <c r="T35" s="46"/>
-      <c r="U35" s="46"/>
-    </row>
-    <row r="36" spans="2:21" ht="39.6" customHeight="1" x14ac:dyDescent="0.25">
+    </row>
+    <row r="36" spans="2:20" ht="39.6" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="L36" s="46"/>
       <c r="M36" s="46"/>
       <c r="N36" s="46"/>
       <c r="O36" s="46"/>
@@ -1551,9 +1555,8 @@
       <c r="R36" s="46"/>
       <c r="S36" s="46"/>
       <c r="T36" s="46"/>
-      <c r="U36" s="46"/>
-    </row>
-    <row r="37" spans="2:21" x14ac:dyDescent="0.25">
+    </row>
+    <row r="37" spans="2:20" x14ac:dyDescent="0.25">
       <c r="B37" s="43"/>
       <c r="C37" s="43"/>
       <c r="D37" s="43"/>
@@ -1564,7 +1567,7 @@
       <c r="I37" s="43"/>
       <c r="J37" s="43"/>
     </row>
-    <row r="38" spans="2:21" x14ac:dyDescent="0.25">
+    <row r="38" spans="2:20" x14ac:dyDescent="0.25">
       <c r="B38" s="44"/>
       <c r="C38" s="44"/>
       <c r="D38" s="44"/>
@@ -1575,7 +1578,7 @@
       <c r="I38" s="44"/>
       <c r="J38" s="44"/>
     </row>
-    <row r="39" spans="2:21" x14ac:dyDescent="0.25">
+    <row r="39" spans="2:20" x14ac:dyDescent="0.25">
       <c r="B39" s="44"/>
       <c r="C39" s="44"/>
       <c r="D39" s="44"/>
@@ -1586,15 +1589,15 @@
       <c r="I39" s="44"/>
       <c r="J39" s="44"/>
     </row>
-    <row r="44" spans="2:21" ht="58.15" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="46" spans="2:21" ht="59.45" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="44" spans="2:20" ht="58.15" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="46" spans="2:20" ht="59.45" customHeight="1" x14ac:dyDescent="0.25"/>
   </sheetData>
   <mergeCells count="21">
     <mergeCell ref="B37:J37"/>
     <mergeCell ref="B38:J38"/>
     <mergeCell ref="B39:J39"/>
-    <mergeCell ref="M11:U16"/>
-    <mergeCell ref="M25:U36"/>
+    <mergeCell ref="L11:T16"/>
+    <mergeCell ref="L25:T36"/>
     <mergeCell ref="A4:J4"/>
     <mergeCell ref="A5:J5"/>
     <mergeCell ref="B10:J10"/>

</xml_diff>

<commit_message>
Update binary files for exporter and formato templates; ensure compatibility with recent changes
</commit_message>
<xml_diff>
--- a/templates/formato.xlsx
+++ b/templates/formato.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/e039d0c270e9facf/Desktop/Developer/UANL---LABORATORIO-DE-ALIMENTOS-MEDICAMENTOS-Y-TOXICOLOGIA/templates/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="283" documentId="8_{47FAC42F-AC07-43D6-8172-01CEADEBF0F6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{AB47CCD7-2A7F-430E-B7B5-7AC47D685782}"/>
+  <xr:revisionPtr revIDLastSave="301" documentId="8_{47FAC42F-AC07-43D6-8172-01CEADEBF0F6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{3BC55181-E269-40E1-9B6D-A71206931ECF}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{1CB8A4CE-E91B-448F-9BE6-E546BA7C8907}"/>
+    <workbookView xWindow="-23148" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{1CB8A4CE-E91B-448F-9BE6-E546BA7C8907}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -507,9 +507,9 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>10</xdr:col>
-      <xdr:colOff>19050</xdr:colOff>
+      <xdr:colOff>34290</xdr:colOff>
       <xdr:row>5</xdr:row>
-      <xdr:rowOff>58947</xdr:rowOff>
+      <xdr:rowOff>72282</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -568,7 +568,7 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>11</xdr:col>
-      <xdr:colOff>216072</xdr:colOff>
+      <xdr:colOff>225597</xdr:colOff>
       <xdr:row>40</xdr:row>
       <xdr:rowOff>186690</xdr:rowOff>
     </xdr:to>
@@ -628,8 +628,8 @@
       <xdr:rowOff>1</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>20</xdr:col>
-      <xdr:colOff>140865</xdr:colOff>
+      <xdr:col>21</xdr:col>
+      <xdr:colOff>346605</xdr:colOff>
       <xdr:row>5</xdr:row>
       <xdr:rowOff>38101</xdr:rowOff>
     </xdr:to>
@@ -1005,7 +1005,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{677BF1A9-BE92-4F6B-8063-3CDF98601680}">
-  <dimension ref="A4:T46"/>
+  <dimension ref="A4:U46"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="3.7109375" customWidth="1"/>
@@ -1019,13 +1019,16 @@
     <col min="10" max="10" width="3.85546875" customWidth="1"/>
     <col min="11" max="11" width="4.85546875" customWidth="1"/>
     <col min="12" max="12" width="9.42578125" customWidth="1"/>
+    <col min="13" max="13" width="3.85546875" customWidth="1"/>
     <col min="14" max="14" width="7.85546875" customWidth="1"/>
+    <col min="15" max="15" width="4.140625" customWidth="1"/>
     <col min="16" max="16" width="8.7109375" customWidth="1"/>
-    <col min="18" max="18" width="4.140625" customWidth="1"/>
-    <col min="19" max="19" width="5" customWidth="1"/>
+    <col min="17" max="17" width="3.5703125" customWidth="1"/>
+    <col min="18" max="18" width="8.85546875" customWidth="1"/>
+    <col min="19" max="19" width="4.28515625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="4" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A4" s="29"/>
       <c r="B4" s="29"/>
       <c r="C4" s="29"/>
@@ -1037,7 +1040,7 @@
       <c r="I4" s="29"/>
       <c r="J4" s="29"/>
     </row>
-    <row r="5" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A5" s="29"/>
       <c r="B5" s="29"/>
       <c r="C5" s="29"/>
@@ -1049,7 +1052,7 @@
       <c r="I5" s="29"/>
       <c r="J5" s="29"/>
     </row>
-    <row r="6" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A6" s="1"/>
       <c r="B6" s="1"/>
       <c r="C6" s="1"/>
@@ -1061,7 +1064,7 @@
       <c r="I6" s="1"/>
       <c r="J6" s="1"/>
     </row>
-    <row r="7" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A7" s="1"/>
       <c r="B7" s="1"/>
       <c r="C7" s="1"/>
@@ -1073,7 +1076,7 @@
       <c r="I7" s="1"/>
       <c r="J7" s="1"/>
     </row>
-    <row r="8" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:21" x14ac:dyDescent="0.25">
       <c r="B8" s="19" t="s">
         <v>18</v>
       </c>
@@ -1089,7 +1092,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="10" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:21" x14ac:dyDescent="0.25">
       <c r="B10" s="30" t="s">
         <v>0</v>
       </c>
@@ -1105,7 +1108,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="11" spans="1:20" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:21" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="L11" s="45" t="s">
         <v>21</v>
       </c>
@@ -1117,8 +1120,9 @@
       <c r="R11" s="45"/>
       <c r="S11" s="45"/>
       <c r="T11" s="45"/>
-    </row>
-    <row r="12" spans="1:20" x14ac:dyDescent="0.25">
+      <c r="U11" s="45"/>
+    </row>
+    <row r="12" spans="1:21" x14ac:dyDescent="0.25">
       <c r="B12" s="42" t="s">
         <v>17</v>
       </c>
@@ -1134,8 +1138,9 @@
       <c r="R12" s="45"/>
       <c r="S12" s="45"/>
       <c r="T12" s="45"/>
-    </row>
-    <row r="13" spans="1:20" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="U12" s="45"/>
+    </row>
+    <row r="13" spans="1:21" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="L13" s="45"/>
       <c r="M13" s="45"/>
       <c r="N13" s="45"/>
@@ -1145,8 +1150,9 @@
       <c r="R13" s="45"/>
       <c r="S13" s="45"/>
       <c r="T13" s="45"/>
-    </row>
-    <row r="14" spans="1:20" x14ac:dyDescent="0.25">
+      <c r="U13" s="45"/>
+    </row>
+    <row r="14" spans="1:21" x14ac:dyDescent="0.25">
       <c r="B14" s="5"/>
       <c r="C14" s="6"/>
       <c r="D14" s="6"/>
@@ -1165,8 +1171,9 @@
       <c r="R14" s="45"/>
       <c r="S14" s="45"/>
       <c r="T14" s="45"/>
-    </row>
-    <row r="15" spans="1:20" ht="21" x14ac:dyDescent="0.35">
+      <c r="U14" s="45"/>
+    </row>
+    <row r="15" spans="1:21" ht="21" x14ac:dyDescent="0.35">
       <c r="B15" s="39" t="s">
         <v>9</v>
       </c>
@@ -1187,8 +1194,9 @@
       <c r="R15" s="45"/>
       <c r="S15" s="45"/>
       <c r="T15" s="45"/>
-    </row>
-    <row r="16" spans="1:20" x14ac:dyDescent="0.25">
+      <c r="U15" s="45"/>
+    </row>
+    <row r="16" spans="1:21" x14ac:dyDescent="0.25">
       <c r="B16" s="3"/>
       <c r="J16" s="4"/>
       <c r="L16" s="45"/>
@@ -1200,8 +1208,9 @@
       <c r="R16" s="45"/>
       <c r="S16" s="45"/>
       <c r="T16" s="45"/>
-    </row>
-    <row r="17" spans="2:20" x14ac:dyDescent="0.25">
+      <c r="U16" s="45"/>
+    </row>
+    <row r="17" spans="2:21" x14ac:dyDescent="0.25">
       <c r="B17" s="3"/>
       <c r="C17" s="20" t="s">
         <v>14</v>
@@ -1214,7 +1223,7 @@
       <c r="I17" s="10"/>
       <c r="J17" s="4"/>
     </row>
-    <row r="18" spans="2:20" x14ac:dyDescent="0.25">
+    <row r="18" spans="2:21" x14ac:dyDescent="0.25">
       <c r="B18" s="3"/>
       <c r="C18" s="20" t="s">
         <v>15</v>
@@ -1226,7 +1235,7 @@
       <c r="I18" s="10"/>
       <c r="J18" s="4"/>
     </row>
-    <row r="19" spans="2:20" x14ac:dyDescent="0.25">
+    <row r="19" spans="2:21" x14ac:dyDescent="0.25">
       <c r="B19" s="3"/>
       <c r="C19" s="21" t="s">
         <v>16</v>
@@ -1239,7 +1248,7 @@
       <c r="I19" s="12"/>
       <c r="J19" s="4"/>
     </row>
-    <row r="20" spans="2:20" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="20" spans="2:21" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B20" s="3"/>
       <c r="C20" s="10"/>
       <c r="D20" s="10"/>
@@ -1259,7 +1268,7 @@
       <c r="P20" s="28"/>
       <c r="Q20" s="28"/>
     </row>
-    <row r="21" spans="2:20" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="21" spans="2:21" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B21" s="3"/>
       <c r="C21" s="37" t="s">
         <v>2</v>
@@ -1279,7 +1288,7 @@
       <c r="R21" s="28"/>
       <c r="S21" s="28"/>
     </row>
-    <row r="22" spans="2:20" x14ac:dyDescent="0.25">
+    <row r="22" spans="2:21" x14ac:dyDescent="0.25">
       <c r="B22" s="3"/>
       <c r="C22" s="36" t="s">
         <v>3</v>
@@ -1300,7 +1309,7 @@
       <c r="R22" s="28"/>
       <c r="S22" s="28"/>
     </row>
-    <row r="23" spans="2:20" x14ac:dyDescent="0.25">
+    <row r="23" spans="2:21" x14ac:dyDescent="0.25">
       <c r="B23" s="3"/>
       <c r="C23" s="36" t="s">
         <v>4</v>
@@ -1321,7 +1330,7 @@
       <c r="R23" s="28"/>
       <c r="S23" s="28"/>
     </row>
-    <row r="24" spans="2:20" x14ac:dyDescent="0.25">
+    <row r="24" spans="2:21" x14ac:dyDescent="0.25">
       <c r="B24" s="3"/>
       <c r="C24" s="30" t="s">
         <v>10</v>
@@ -1341,7 +1350,7 @@
       <c r="R24" s="28"/>
       <c r="S24" s="28"/>
     </row>
-    <row r="25" spans="2:20" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="25" spans="2:21" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B25" s="3"/>
       <c r="C25" s="30" t="s">
         <v>11</v>
@@ -1363,8 +1372,9 @@
       <c r="R25" s="46"/>
       <c r="S25" s="46"/>
       <c r="T25" s="46"/>
-    </row>
-    <row r="26" spans="2:20" x14ac:dyDescent="0.25">
+      <c r="U25" s="46"/>
+    </row>
+    <row r="26" spans="2:21" x14ac:dyDescent="0.25">
       <c r="B26" s="3"/>
       <c r="C26" s="38" t="s">
         <v>5</v>
@@ -1385,8 +1395,9 @@
       <c r="R26" s="46"/>
       <c r="S26" s="46"/>
       <c r="T26" s="46"/>
-    </row>
-    <row r="27" spans="2:20" x14ac:dyDescent="0.25">
+      <c r="U26" s="46"/>
+    </row>
+    <row r="27" spans="2:21" x14ac:dyDescent="0.25">
       <c r="B27" s="3"/>
       <c r="C27" s="35" t="s">
         <v>12</v>
@@ -1405,8 +1416,9 @@
       <c r="R27" s="46"/>
       <c r="S27" s="46"/>
       <c r="T27" s="46"/>
-    </row>
-    <row r="28" spans="2:20" x14ac:dyDescent="0.25">
+      <c r="U27" s="46"/>
+    </row>
+    <row r="28" spans="2:21" x14ac:dyDescent="0.25">
       <c r="B28" s="3"/>
       <c r="C28" s="13" t="s">
         <v>13</v>
@@ -1425,8 +1437,9 @@
       <c r="R28" s="46"/>
       <c r="S28" s="46"/>
       <c r="T28" s="46"/>
-    </row>
-    <row r="29" spans="2:20" x14ac:dyDescent="0.25">
+      <c r="U28" s="46"/>
+    </row>
+    <row r="29" spans="2:21" x14ac:dyDescent="0.25">
       <c r="B29" s="3"/>
       <c r="C29" s="36" t="s">
         <v>6</v>
@@ -1447,8 +1460,9 @@
       <c r="R29" s="46"/>
       <c r="S29" s="46"/>
       <c r="T29" s="46"/>
-    </row>
-    <row r="30" spans="2:20" x14ac:dyDescent="0.25">
+      <c r="U29" s="46"/>
+    </row>
+    <row r="30" spans="2:21" x14ac:dyDescent="0.25">
       <c r="B30" s="3"/>
       <c r="C30" s="37" t="s">
         <v>7</v>
@@ -1469,8 +1483,9 @@
       <c r="R30" s="46"/>
       <c r="S30" s="46"/>
       <c r="T30" s="46"/>
-    </row>
-    <row r="31" spans="2:20" x14ac:dyDescent="0.25">
+      <c r="U30" s="46"/>
+    </row>
+    <row r="31" spans="2:21" x14ac:dyDescent="0.25">
       <c r="B31" s="3"/>
       <c r="C31" s="10"/>
       <c r="D31" s="10"/>
@@ -1489,8 +1504,9 @@
       <c r="R31" s="46"/>
       <c r="S31" s="46"/>
       <c r="T31" s="46"/>
-    </row>
-    <row r="32" spans="2:20" ht="31.9" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="U31" s="46"/>
+    </row>
+    <row r="32" spans="2:21" ht="31.9" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B32" s="31" t="s">
         <v>8</v>
       </c>
@@ -1511,8 +1527,9 @@
       <c r="R32" s="46"/>
       <c r="S32" s="46"/>
       <c r="T32" s="46"/>
-    </row>
-    <row r="33" spans="2:20" x14ac:dyDescent="0.25">
+      <c r="U32" s="46"/>
+    </row>
+    <row r="33" spans="2:21" x14ac:dyDescent="0.25">
       <c r="L33" s="46"/>
       <c r="M33" s="46"/>
       <c r="N33" s="46"/>
@@ -1522,8 +1539,9 @@
       <c r="R33" s="46"/>
       <c r="S33" s="46"/>
       <c r="T33" s="46"/>
-    </row>
-    <row r="34" spans="2:20" x14ac:dyDescent="0.25">
+      <c r="U33" s="46"/>
+    </row>
+    <row r="34" spans="2:21" x14ac:dyDescent="0.25">
       <c r="L34" s="46"/>
       <c r="M34" s="46"/>
       <c r="N34" s="46"/>
@@ -1533,8 +1551,9 @@
       <c r="R34" s="46"/>
       <c r="S34" s="46"/>
       <c r="T34" s="46"/>
-    </row>
-    <row r="35" spans="2:20" x14ac:dyDescent="0.25">
+      <c r="U34" s="46"/>
+    </row>
+    <row r="35" spans="2:21" x14ac:dyDescent="0.25">
       <c r="L35" s="46"/>
       <c r="M35" s="46"/>
       <c r="N35" s="46"/>
@@ -1544,8 +1563,9 @@
       <c r="R35" s="46"/>
       <c r="S35" s="46"/>
       <c r="T35" s="46"/>
-    </row>
-    <row r="36" spans="2:20" ht="39.6" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="U35" s="46"/>
+    </row>
+    <row r="36" spans="2:21" ht="39.6" customHeight="1" x14ac:dyDescent="0.25">
       <c r="L36" s="46"/>
       <c r="M36" s="46"/>
       <c r="N36" s="46"/>
@@ -1555,8 +1575,9 @@
       <c r="R36" s="46"/>
       <c r="S36" s="46"/>
       <c r="T36" s="46"/>
-    </row>
-    <row r="37" spans="2:20" x14ac:dyDescent="0.25">
+      <c r="U36" s="46"/>
+    </row>
+    <row r="37" spans="2:21" x14ac:dyDescent="0.25">
       <c r="B37" s="43"/>
       <c r="C37" s="43"/>
       <c r="D37" s="43"/>
@@ -1567,7 +1588,7 @@
       <c r="I37" s="43"/>
       <c r="J37" s="43"/>
     </row>
-    <row r="38" spans="2:20" x14ac:dyDescent="0.25">
+    <row r="38" spans="2:21" x14ac:dyDescent="0.25">
       <c r="B38" s="44"/>
       <c r="C38" s="44"/>
       <c r="D38" s="44"/>
@@ -1578,7 +1599,7 @@
       <c r="I38" s="44"/>
       <c r="J38" s="44"/>
     </row>
-    <row r="39" spans="2:20" x14ac:dyDescent="0.25">
+    <row r="39" spans="2:21" x14ac:dyDescent="0.25">
       <c r="B39" s="44"/>
       <c r="C39" s="44"/>
       <c r="D39" s="44"/>
@@ -1589,15 +1610,15 @@
       <c r="I39" s="44"/>
       <c r="J39" s="44"/>
     </row>
-    <row r="44" spans="2:20" ht="58.15" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="46" spans="2:20" ht="59.45" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="44" spans="2:21" ht="58.15" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="46" spans="2:21" ht="59.45" customHeight="1" x14ac:dyDescent="0.25"/>
   </sheetData>
   <mergeCells count="21">
     <mergeCell ref="B37:J37"/>
     <mergeCell ref="B38:J38"/>
     <mergeCell ref="B39:J39"/>
-    <mergeCell ref="L11:T16"/>
-    <mergeCell ref="L25:T36"/>
+    <mergeCell ref="L11:U16"/>
+    <mergeCell ref="L25:U36"/>
     <mergeCell ref="A4:J4"/>
     <mergeCell ref="A5:J5"/>
     <mergeCell ref="B10:J10"/>

</xml_diff>